<commit_message>
Tuned and working version of concept_control
</commit_message>
<xml_diff>
--- a/Sizing/concepts_tabulations.xlsx
+++ b/Sizing/concepts_tabulations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8522608F-7DE1-4296-8745-1C6D1FB317F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E662352-9A24-4E63-A31D-6E5EF25FFA53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="132">
   <si>
     <t>Deliverable</t>
   </si>
@@ -56,21 +56,9 @@
     <t>Performance</t>
   </si>
   <si>
-    <t>CV Landing dist. limit</t>
-  </si>
-  <si>
     <t>Max L/D</t>
   </si>
   <si>
-    <t>Supercruise speed</t>
-  </si>
-  <si>
-    <t>Supercruise Range</t>
-  </si>
-  <si>
-    <t>Sortie Ranges</t>
-  </si>
-  <si>
     <t>Notes</t>
   </si>
   <si>
@@ -221,9 +209,6 @@
     <t>Wing Area [m2]</t>
   </si>
   <si>
-    <t>CV approach limit</t>
-  </si>
-  <si>
     <t>F/A-18E</t>
   </si>
   <si>
@@ -260,12 +245,6 @@
     <t>2</t>
   </si>
   <si>
-    <t>65436.8948</t>
-  </si>
-  <si>
-    <t>33158.8948</t>
-  </si>
-  <si>
     <t>3.5672</t>
   </si>
   <si>
@@ -305,30 +284,6 @@
     <t>184.2067</t>
   </si>
   <si>
-    <t>45.4742</t>
-  </si>
-  <si>
-    <t>83.656</t>
-  </si>
-  <si>
-    <t>13.483</t>
-  </si>
-  <si>
-    <t>1870.9863</t>
-  </si>
-  <si>
-    <t>300.7228</t>
-  </si>
-  <si>
-    <t>7150.928</t>
-  </si>
-  <si>
-    <t>0.63284</t>
-  </si>
-  <si>
-    <t>6.4173</t>
-  </si>
-  <si>
     <t>Unit Cost [millions]</t>
   </si>
   <si>
@@ -350,18 +305,12 @@
     <t>Landing Speed [kt]</t>
   </si>
   <si>
-    <t>Uses 1.3x stall</t>
-  </si>
-  <si>
     <t>73.6832</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t>137.1499</t>
-  </si>
-  <si>
     <t>0.3193</t>
   </si>
   <si>
@@ -389,40 +338,100 @@
     <t>45 ton MTOW</t>
   </si>
   <si>
-    <t>1.628</t>
-  </si>
-  <si>
-    <t>8544.2942</t>
-  </si>
-  <si>
-    <t>-0.054139</t>
-  </si>
-  <si>
-    <t>0.071875</t>
-  </si>
-  <si>
-    <t>-0.16595</t>
-  </si>
-  <si>
     <t>-0.3411</t>
   </si>
   <si>
-    <t>-0.27292</t>
-  </si>
-  <si>
-    <t>1142.2424</t>
-  </si>
-  <si>
-    <t>476.3651</t>
-  </si>
-  <si>
-    <t>1249.1855</t>
-  </si>
-  <si>
-    <t>-8531.5937</t>
-  </si>
-  <si>
-    <t>0.29988</t>
+    <t>6500.8437</t>
+  </si>
+  <si>
+    <t>0.69613</t>
+  </si>
+  <si>
+    <t>59488.0861</t>
+  </si>
+  <si>
+    <t>-0.33902</t>
+  </si>
+  <si>
+    <t>23900.0861</t>
+  </si>
+  <si>
+    <t>732.9451</t>
+  </si>
+  <si>
+    <t>505.5753</t>
+  </si>
+  <si>
+    <t>911.1361</t>
+  </si>
+  <si>
+    <t>6.6602</t>
+  </si>
+  <si>
+    <t>8 Deg/s Sustained Turn</t>
+  </si>
+  <si>
+    <t>Max Sustained Turn Rate [deg/s]</t>
+  </si>
+  <si>
+    <t>0.062744</t>
+  </si>
+  <si>
+    <t>Landing SEROC</t>
+  </si>
+  <si>
+    <t>Landing SEROC [ft/min]</t>
+  </si>
+  <si>
+    <t>1.6589</t>
+  </si>
+  <si>
+    <t>53.7409</t>
+  </si>
+  <si>
+    <t>130.6523</t>
+  </si>
+  <si>
+    <t>1691.3094</t>
+  </si>
+  <si>
+    <t>272.8649</t>
+  </si>
+  <si>
+    <t>607.4833</t>
+  </si>
+  <si>
+    <t>-4337.0929</t>
+  </si>
+  <si>
+    <t>0.15245</t>
+  </si>
+  <si>
+    <t>-0.18249</t>
+  </si>
+  <si>
+    <t>-0.1089</t>
+  </si>
+  <si>
+    <t>28.4223</t>
+  </si>
+  <si>
+    <t>16.5467</t>
+  </si>
+  <si>
+    <t>Uses 1.3x stall (this is at MTOW)</t>
+  </si>
+  <si>
+    <t>145.3531</t>
+  </si>
+  <si>
+    <t>1298.9508</t>
+  </si>
+  <si>
+    <t>0.0024352</t>
+  </si>
+  <si>
+    <t>-1.5979</t>
   </si>
 </sst>
 </file>
@@ -979,7 +988,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="38.77734375" customWidth="1"/>
@@ -994,16 +1003,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -1015,7 +1024,7 @@
         <v>4</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -1033,10 +1042,10 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="12"/>
@@ -1045,15 +1054,15 @@
       <c r="G3" s="12"/>
       <c r="H3" s="13"/>
       <c r="I3" s="8" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="12"/>
@@ -1062,15 +1071,15 @@
       <c r="G4" s="12"/>
       <c r="H4" s="13"/>
       <c r="I4" s="8" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="12"/>
@@ -1079,15 +1088,15 @@
       <c r="G5" s="12"/>
       <c r="H5" s="13"/>
       <c r="I5" s="8" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C6" s="11"/>
       <c r="D6" s="12"/>
@@ -1096,15 +1105,15 @@
       <c r="G6" s="12"/>
       <c r="H6" s="13"/>
       <c r="I6" s="8" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C7" s="11"/>
       <c r="D7" s="12"/>
@@ -1113,15 +1122,15 @@
       <c r="G7" s="12"/>
       <c r="H7" s="13"/>
       <c r="I7" s="8" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="C8" s="11"/>
       <c r="D8" s="12"/>
@@ -1130,14 +1139,16 @@
       <c r="G8" s="12"/>
       <c r="H8" s="13"/>
       <c r="I8" s="8" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B9" s="11"/>
+        <v>36</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>116</v>
+      </c>
       <c r="C9" s="11"/>
       <c r="D9" s="12"/>
       <c r="E9" s="12"/>
@@ -1148,9 +1159,11 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="11"/>
+        <v>37</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C10" s="11"/>
       <c r="D10" s="12"/>
       <c r="E10" s="12"/>
@@ -1161,10 +1174,10 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>40</v>
+        <v>114</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>89</v>
+        <v>129</v>
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="12"/>
@@ -1176,10 +1189,10 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>90</v>
+        <v>125</v>
       </c>
       <c r="C12" s="11"/>
       <c r="D12" s="12"/>
@@ -1191,10 +1204,10 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>42</v>
+        <v>111</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>91</v>
+        <v>126</v>
       </c>
       <c r="C13" s="11"/>
       <c r="D13" s="12"/>
@@ -1206,10 +1219,10 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>92</v>
+        <v>118</v>
       </c>
       <c r="C14" s="11"/>
       <c r="D14" s="12"/>
@@ -1218,15 +1231,15 @@
       <c r="G14" s="12"/>
       <c r="H14" s="12"/>
       <c r="I14" s="9" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>93</v>
+        <v>119</v>
       </c>
       <c r="C15" s="11"/>
       <c r="D15" s="12"/>
@@ -1235,15 +1248,15 @@
       <c r="G15" s="12"/>
       <c r="H15" s="12"/>
       <c r="I15" s="9" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="C16" s="11"/>
       <c r="D16" s="12"/>
@@ -1255,10 +1268,10 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
       <c r="C17" s="11"/>
       <c r="D17" s="12"/>
@@ -1270,10 +1283,10 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>126</v>
+        <v>108</v>
       </c>
       <c r="C18" s="11"/>
       <c r="D18" s="12"/>
@@ -1285,10 +1298,10 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C19" s="11"/>
       <c r="D19" s="12"/>
@@ -1300,10 +1313,10 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="C20" s="11"/>
       <c r="D20" s="12"/>
@@ -1315,10 +1328,10 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="C21" s="11"/>
       <c r="D21" s="12"/>
@@ -1327,15 +1340,15 @@
       <c r="G21" s="12"/>
       <c r="H21" s="12"/>
       <c r="I21" s="9" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="C22" s="11"/>
       <c r="D22" s="12"/>
@@ -1344,15 +1357,15 @@
       <c r="G22" s="12"/>
       <c r="H22" s="12"/>
       <c r="I22" s="9" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="C23" s="11"/>
       <c r="D23" s="12"/>
@@ -1361,86 +1374,100 @@
       <c r="G23" s="12"/>
       <c r="H23" s="12"/>
       <c r="I23" s="9" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="12"/>
-      <c r="I24" s="9"/>
+      <c r="A24" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="10"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="11"/>
+      <c r="B25" s="11" t="s">
+        <v>58</v>
+      </c>
       <c r="C25" s="11"/>
-      <c r="D25" s="12"/>
+      <c r="D25" s="12" t="s">
+        <v>74</v>
+      </c>
       <c r="E25" s="12"/>
       <c r="F25" s="12"/>
       <c r="G25" s="12"/>
       <c r="H25" s="12"/>
-      <c r="I25" s="9"/>
+      <c r="I25" s="9" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B26" s="11"/>
+        <v>11</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>59</v>
+      </c>
       <c r="C26" s="11"/>
       <c r="D26" s="12"/>
       <c r="E26" s="12"/>
       <c r="F26" s="12"/>
       <c r="G26" s="12"/>
       <c r="H26" s="12"/>
-      <c r="I26" s="9"/>
+      <c r="I26" s="9" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="15"/>
-      <c r="G27" s="15"/>
-      <c r="H27" s="15"/>
-      <c r="I27" s="10"/>
+      <c r="A27" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="11"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="9" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C28" s="11"/>
       <c r="D28" s="12" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="E28" s="12"/>
       <c r="F28" s="12"/>
       <c r="G28" s="12"/>
       <c r="H28" s="12"/>
       <c r="I28" s="9" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C29" s="11"/>
       <c r="D29" s="12"/>
@@ -1449,15 +1476,15 @@
       <c r="G29" s="12"/>
       <c r="H29" s="12"/>
       <c r="I29" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C30" s="11"/>
       <c r="D30" s="12"/>
@@ -1466,34 +1493,30 @@
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="9" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C31" s="11"/>
-      <c r="D31" s="12" t="s">
-        <v>82</v>
-      </c>
+      <c r="D31" s="12"/>
       <c r="E31" s="12"/>
       <c r="F31" s="12"/>
       <c r="G31" s="12"/>
       <c r="H31" s="12"/>
-      <c r="I31" s="9" t="s">
-        <v>20</v>
-      </c>
+      <c r="I31" s="9"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C32" s="11"/>
       <c r="D32" s="12"/>
@@ -1502,15 +1525,15 @@
       <c r="G32" s="12"/>
       <c r="H32" s="12"/>
       <c r="I32" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C33" s="11"/>
       <c r="D33" s="12"/>
@@ -1519,15 +1542,15 @@
       <c r="G33" s="12"/>
       <c r="H33" s="12"/>
       <c r="I33" s="9" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C34" s="11"/>
       <c r="D34" s="12"/>
@@ -1539,10 +1562,10 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>23</v>
+        <v>86</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="C35" s="11"/>
       <c r="D35" s="12"/>
@@ -1551,15 +1574,15 @@
       <c r="G35" s="12"/>
       <c r="H35" s="12"/>
       <c r="I35" s="9" t="s">
-        <v>24</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="C36" s="11"/>
       <c r="D36" s="12"/>
@@ -1568,15 +1591,15 @@
       <c r="G36" s="12"/>
       <c r="H36" s="12"/>
       <c r="I36" s="9" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C37" s="11"/>
       <c r="D37" s="12"/>
@@ -1587,28 +1610,24 @@
       <c r="I37" s="9"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A38" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="B38" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="C38" s="11"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
-      <c r="F38" s="12"/>
-      <c r="G38" s="12"/>
-      <c r="H38" s="12"/>
-      <c r="I38" s="9" t="s">
-        <v>102</v>
-      </c>
+      <c r="A38" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B38" s="15"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="15"/>
+      <c r="G38" s="15"/>
+      <c r="H38" s="15"/>
+      <c r="I38" s="10"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>33</v>
+        <v>103</v>
       </c>
       <c r="C39" s="11"/>
       <c r="D39" s="12"/>
@@ -1616,59 +1635,59 @@
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
       <c r="H39" s="12"/>
-      <c r="I39" s="9" t="s">
-        <v>34</v>
-      </c>
+      <c r="I39" s="9"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="C40" s="11"/>
-      <c r="D40" s="12"/>
-      <c r="E40" s="12"/>
-      <c r="F40" s="12"/>
-      <c r="G40" s="12"/>
+        <v>105</v>
+      </c>
+      <c r="C40" s="14"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="13"/>
+      <c r="F40" s="13"/>
+      <c r="G40" s="13"/>
       <c r="H40" s="12"/>
       <c r="I40" s="9"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B41" s="15"/>
-      <c r="C41" s="15"/>
-      <c r="D41" s="15"/>
-      <c r="E41" s="15"/>
-      <c r="F41" s="15"/>
-      <c r="G41" s="15"/>
-      <c r="H41" s="15"/>
-      <c r="I41" s="10"/>
+      <c r="A41" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C41" s="14"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="9"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="C42" s="11"/>
-      <c r="D42" s="12"/>
-      <c r="E42" s="12"/>
-      <c r="F42" s="12"/>
-      <c r="G42" s="12"/>
+        <v>70</v>
+      </c>
+      <c r="C42" s="14"/>
+      <c r="D42" s="13"/>
+      <c r="E42" s="13"/>
+      <c r="F42" s="13"/>
+      <c r="G42" s="13"/>
       <c r="H42" s="12"/>
       <c r="I42" s="9"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C43" s="14"/>
       <c r="D43" s="13"/>
@@ -1683,7 +1702,7 @@
         <v>54</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C44" s="14"/>
       <c r="D44" s="13"/>
@@ -1695,10 +1714,10 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C45" s="14"/>
       <c r="D45" s="13"/>
@@ -1709,41 +1728,41 @@
       <c r="I45" s="9"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="B46" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="C46" s="14"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="13"/>
-      <c r="F46" s="13"/>
-      <c r="G46" s="13"/>
-      <c r="H46" s="12"/>
-      <c r="I46" s="9"/>
+      <c r="A46" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B46" s="15"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="15"/>
+      <c r="H46" s="15"/>
+      <c r="I46" s="10"/>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="C47" s="14"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13"/>
-      <c r="F47" s="13"/>
-      <c r="G47" s="13"/>
+        <v>122</v>
+      </c>
+      <c r="C47" s="11"/>
+      <c r="D47" s="12"/>
+      <c r="E47" s="12"/>
+      <c r="F47" s="12"/>
+      <c r="G47" s="12"/>
       <c r="H47" s="12"/>
-      <c r="I47" s="9"/>
+      <c r="I47" s="9" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
-        <v>60</v>
+        <v>94</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>80</v>
+        <v>130</v>
       </c>
       <c r="C48" s="14"/>
       <c r="D48" s="13"/>
@@ -1754,41 +1773,41 @@
       <c r="I48" s="9"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A49" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="B49" s="15"/>
-      <c r="C49" s="15"/>
-      <c r="D49" s="15"/>
-      <c r="E49" s="15"/>
-      <c r="F49" s="15"/>
-      <c r="G49" s="15"/>
-      <c r="H49" s="15"/>
-      <c r="I49" s="10" t="s">
+      <c r="A49" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B49" s="11" t="s">
         <v>112</v>
       </c>
+      <c r="C49" s="14"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="13"/>
+      <c r="F49" s="13"/>
+      <c r="G49" s="13"/>
+      <c r="H49" s="12"/>
+      <c r="I49" s="9"/>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="C50" s="11"/>
-      <c r="D50" s="12"/>
-      <c r="E50" s="12"/>
-      <c r="F50" s="12"/>
-      <c r="G50" s="12"/>
+        <v>123</v>
+      </c>
+      <c r="C50" s="14"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="13"/>
+      <c r="F50" s="13"/>
+      <c r="G50" s="13"/>
       <c r="H50" s="12"/>
       <c r="I50" s="9"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>119</v>
+        <v>100</v>
       </c>
       <c r="C51" s="14"/>
       <c r="D51" s="13"/>
@@ -1800,10 +1819,10 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="C52" s="14"/>
       <c r="D52" s="13"/>
@@ -1815,10 +1834,10 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C53" s="14"/>
       <c r="D53" s="13"/>
@@ -1826,14 +1845,13 @@
       <c r="F53" s="13"/>
       <c r="G53" s="13"/>
       <c r="H53" s="12"/>
-      <c r="I53" s="9"/>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="C54" s="14"/>
       <c r="D54" s="13"/>
@@ -1841,22 +1859,6 @@
       <c r="F54" s="13"/>
       <c r="G54" s="13"/>
       <c r="H54" s="12"/>
-      <c r="I54" s="9"/>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A55" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="B55" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="C55" s="14"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="13"/>
-      <c r="F55" s="13"/>
-      <c r="G55" s="13"/>
-      <c r="H55" s="12"/>
-      <c r="I55" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1865,25 +1867,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100841FCFF63B2DEE4FAB3ABDCB2B58E191" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6537ae6c172b48d8001feb3057ef3193">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f38bd768-81b4-450c-b73d-1a8fa3ba2722" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e79d1da23033c2d9c1658a7b9c3763cb" ns2:_="">
     <xsd:import namespace="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
@@ -2055,10 +2038,39 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0D3B35F-2651-4930-8D88-666C35501CF8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2074,19 +2086,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0D3B35F-2651-4930-8D88-666C35501CF8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Working sizing and concept control code
</commit_message>
<xml_diff>
--- a/Sizing/concepts_tabulations.xlsx
+++ b/Sizing/concepts_tabulations.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E662352-9A24-4E63-A31D-6E5EF25FFA53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12514195-5942-4AE4-97F2-7ED29CB638FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
     <sheet name="Concepts" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="true" iterate="true"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="374" uniqueCount="173">
   <si>
     <t>Deliverable</t>
   </si>
@@ -432,13 +432,136 @@
   </si>
   <si>
     <t>-1.5979</t>
+  </si>
+  <si>
+    <t>F/A-18E_Sized</t>
+  </si>
+  <si>
+    <t>F-16</t>
+  </si>
+  <si>
+    <t>732.2682</t>
+  </si>
+  <si>
+    <t>505.8509</t>
+  </si>
+  <si>
+    <t>911.0097</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Temp</t>
+  </si>
+  <si>
+    <t>71.9985</t>
+  </si>
+  <si>
+    <t>2.2969</t>
+  </si>
+  <si>
+    <t>1.6675</t>
+  </si>
+  <si>
+    <t>98.0516</t>
+  </si>
+  <si>
+    <t>63.0246</t>
+  </si>
+  <si>
+    <t>138.2653</t>
+  </si>
+  <si>
+    <t>1304.2817</t>
+  </si>
+  <si>
+    <t>40.6897</t>
+  </si>
+  <si>
+    <t>26.2351</t>
+  </si>
+  <si>
+    <t>2288.2981</t>
+  </si>
+  <si>
+    <t>426.048</t>
+  </si>
+  <si>
+    <t>1115.6452</t>
+  </si>
+  <si>
+    <t>763.9478</t>
+  </si>
+  <si>
+    <t>1309.7927</t>
+  </si>
+  <si>
+    <t>5624.6918</t>
+  </si>
+  <si>
+    <t>5.0621</t>
+  </si>
+  <si>
+    <t>2733.3813</t>
+  </si>
+  <si>
+    <t>0.72081</t>
+  </si>
+  <si>
+    <t>10.1342</t>
+  </si>
+  <si>
+    <t>27600.4439</t>
+  </si>
+  <si>
+    <t>18.2623</t>
+  </si>
+  <si>
+    <t>7.6838</t>
+  </si>
+  <si>
+    <t>2.5552</t>
+  </si>
+  <si>
+    <t>57450.8461</t>
+  </si>
+  <si>
+    <t>22712.4022</t>
+  </si>
+  <si>
+    <t>5.1195</t>
+  </si>
+  <si>
+    <t>93.4938</t>
+  </si>
+  <si>
+    <t>-0.00018341</t>
+  </si>
+  <si>
+    <t>-0.32378</t>
+  </si>
+  <si>
+    <t>-0.18621</t>
+  </si>
+  <si>
+    <t>-0.0014064</t>
+  </si>
+  <si>
+    <t>-0.36166</t>
+  </si>
+  <si>
+    <t>-0.7396</t>
+  </si>
+  <si>
+    <t>-1.6086</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -472,13 +595,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
+        <fgColor theme="4" tint="0.39997558519242"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="0" tint="-0.14999847407453"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -489,7 +612,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -603,57 +726,69 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -672,7 +807,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -823,7 +958,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -847,9 +982,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -873,7 +1008,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -908,7 +1043,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -926,7 +1061,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -951,7 +1086,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -987,18 +1122,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
-  <dimension ref="A1:I54"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
+  <dimension ref="A1:L54"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.77734375" customWidth="1"/>
-    <col min="2" max="2" width="10.44140625" customWidth="1"/>
-    <col min="3" max="3" width="4.6640625" customWidth="1"/>
-    <col min="4" max="8" width="9.77734375" customWidth="1"/>
-    <col min="9" max="9" width="106.77734375" customWidth="1"/>
+    <col min="1" max="1" width="38.796875" customWidth="true"/>
+    <col min="2" max="2" width="10.5" customWidth="true"/>
+    <col min="3" max="3" width="13.5" customWidth="true"/>
+    <col min="4" max="4" width="4.69921875" customWidth="true"/>
+    <col min="6" max="6" width="9.796875" customWidth="true"/>
+    <col min="12" max="12" width="106.796875" customWidth="true"/>
+    <col min="5" max="5" width="4.69921875" customWidth="true"/>
+    <col min="7" max="7" width="9.796875" customWidth="true"/>
+    <col min="8" max="8" width="9.796875" customWidth="true"/>
+    <col min="9" max="9" width="9.796875" customWidth="true"/>
+    <col min="10" max="10" width="9.796875" customWidth="true"/>
+    <col min="11" max="11" width="6" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" ht="15" thickBot="true" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1006,28 +1148,37 @@
         <v>57</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="K1" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="L1" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1038,346 +1189,454 @@
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="7"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="7"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>82</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
+      <c r="C3" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="8" t="s">
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="8" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>84</v>
       </c>
       <c r="B4" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
+      <c r="C4" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="8" t="s">
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="13"/>
+      <c r="K4" s="13"/>
+      <c r="L4" s="8" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
+      <c r="C5" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="8" t="s">
+      <c r="H5" s="12"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13"/>
+      <c r="L5" s="8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>34</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
+      <c r="C6" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="8" t="s">
+      <c r="H6" s="12"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="13"/>
+      <c r="L6" s="8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>31</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
+      <c r="C7" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="8" t="s">
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="8" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>88</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
+      <c r="C8" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="8" t="s">
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13"/>
+      <c r="L8" s="8" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>36</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
+      <c r="C9" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
       <c r="F9" s="12"/>
       <c r="G9" s="12"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="8"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="13"/>
+      <c r="L9" s="8"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>37</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
+      <c r="C10" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="8"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H10" s="12"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="13"/>
+      <c r="L10" s="8"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>114</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
+      <c r="C11" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="8"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="13"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="8"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>38</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
+      <c r="C12" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="8"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="8"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>111</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
+      <c r="C13" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
       <c r="F13" s="12"/>
       <c r="G13" s="12"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="8"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="13"/>
+      <c r="K13" s="13"/>
+      <c r="L13" s="8"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>78</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
+      <c r="C14" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
       <c r="H14" s="12"/>
-      <c r="I14" s="9" t="s">
+      <c r="I14" s="12"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>79</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
+      <c r="C15" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
       <c r="F15" s="12"/>
       <c r="G15" s="12"/>
       <c r="H15" s="12"/>
-      <c r="I15" s="9" t="s">
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>43</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
+      <c r="C16" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
       <c r="H16" s="12"/>
-      <c r="I16" s="9"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>44</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
+      <c r="C17" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
-      <c r="I17" s="9"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>45</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
+      <c r="C18" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
       <c r="F18" s="12"/>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
-      <c r="I18" s="9"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>41</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
+      <c r="C19" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
-      <c r="I19" s="9"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>42</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="C20" s="11"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
+      <c r="C20" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
       <c r="H20" s="12"/>
-      <c r="I20" s="9"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>46</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="C21" s="11"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
+      <c r="C21" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
       <c r="H21" s="12"/>
-      <c r="I21" s="9" t="s">
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>77</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
+      <c r="C22" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
       <c r="H22" s="12"/>
-      <c r="I22" s="9" t="s">
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>6</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="C23" s="11"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
+      <c r="C23" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
       <c r="H23" s="12"/>
-      <c r="I23" s="9" t="s">
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>24</v>
       </c>
@@ -1388,228 +1647,296 @@
       <c r="F24" s="15"/>
       <c r="G24" s="15"/>
       <c r="H24" s="15"/>
-      <c r="I24" s="10"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="15"/>
+      <c r="L24" s="10"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B25" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C25" s="11"/>
-      <c r="D25" s="12" t="s">
+      <c r="C25" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
       <c r="G25" s="12"/>
       <c r="H25" s="12"/>
-      <c r="I25" s="9" t="s">
+      <c r="I25" s="12"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="11"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
+      <c r="C26" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
       <c r="F26" s="12"/>
       <c r="G26" s="12"/>
       <c r="H26" s="12"/>
-      <c r="I26" s="9" t="s">
+      <c r="I26" s="12"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="12"/>
+      <c r="L26" s="9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>13</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="C27" s="11"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
+      <c r="C27" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
       <c r="F27" s="12"/>
       <c r="G27" s="12"/>
       <c r="H27" s="12"/>
-      <c r="I27" s="9" t="s">
+      <c r="I27" s="12"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>15</v>
       </c>
       <c r="B28" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="C28" s="11"/>
-      <c r="D28" s="12" t="s">
+      <c r="C28" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="D28" s="11"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="E28" s="12"/>
-      <c r="F28" s="12"/>
       <c r="G28" s="12"/>
       <c r="H28" s="12"/>
-      <c r="I28" s="9" t="s">
+      <c r="I28" s="12"/>
+      <c r="J28" s="12"/>
+      <c r="K28" s="12"/>
+      <c r="L28" s="9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>17</v>
       </c>
       <c r="B29" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="C29" s="11"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
+      <c r="C29" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="D29" s="11"/>
+      <c r="E29" s="11"/>
       <c r="F29" s="12"/>
       <c r="G29" s="12"/>
       <c r="H29" s="12"/>
-      <c r="I29" s="9" t="s">
+      <c r="I29" s="12"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="12"/>
+      <c r="L29" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B30" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="11"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
+      <c r="C30" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
       <c r="F30" s="12"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
-      <c r="I30" s="9" t="s">
+      <c r="I30" s="12"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="12"/>
+      <c r="L30" s="9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>25</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="11"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
+      <c r="C31" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
       <c r="F31" s="12"/>
       <c r="G31" s="12"/>
       <c r="H31" s="12"/>
-      <c r="I31" s="9"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I31" s="12"/>
+      <c r="J31" s="12"/>
+      <c r="K31" s="12"/>
+      <c r="L31" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>19</v>
       </c>
       <c r="B32" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="C32" s="11"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
+      <c r="C32" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="D32" s="11"/>
+      <c r="E32" s="11"/>
       <c r="F32" s="12"/>
       <c r="G32" s="12"/>
       <c r="H32" s="12"/>
-      <c r="I32" s="9" t="s">
+      <c r="I32" s="12"/>
+      <c r="J32" s="12"/>
+      <c r="K32" s="12"/>
+      <c r="L32" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>21</v>
       </c>
       <c r="B33" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="C33" s="11"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
+      <c r="C33" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="D33" s="11"/>
+      <c r="E33" s="11"/>
       <c r="F33" s="12"/>
       <c r="G33" s="12"/>
       <c r="H33" s="12"/>
-      <c r="I33" s="9" t="s">
+      <c r="I33" s="12"/>
+      <c r="J33" s="12"/>
+      <c r="K33" s="12"/>
+      <c r="L33" s="9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="C34" s="11"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="12"/>
+      <c r="C34" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="D34" s="11"/>
+      <c r="E34" s="11"/>
       <c r="F34" s="12"/>
       <c r="G34" s="12"/>
       <c r="H34" s="12"/>
-      <c r="I34" s="9"/>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I34" s="12"/>
+      <c r="J34" s="12"/>
+      <c r="K34" s="12"/>
+      <c r="L34" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>86</v>
       </c>
       <c r="B35" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="C35" s="11"/>
-      <c r="D35" s="12"/>
-      <c r="E35" s="12"/>
+      <c r="C35" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
       <c r="H35" s="12"/>
-      <c r="I35" s="9" t="s">
+      <c r="I35" s="12"/>
+      <c r="J35" s="12"/>
+      <c r="K35" s="12"/>
+      <c r="L35" s="9" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C36" s="11"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
+      <c r="C36" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
       <c r="F36" s="12"/>
       <c r="G36" s="12"/>
       <c r="H36" s="12"/>
-      <c r="I36" s="9" t="s">
+      <c r="I36" s="12"/>
+      <c r="J36" s="12"/>
+      <c r="K36" s="12"/>
+      <c r="L36" s="9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>52</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="C37" s="11"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="12"/>
+      <c r="C37" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
       <c r="H37" s="12"/>
-      <c r="I37" s="9"/>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I37" s="12"/>
+      <c r="J37" s="12"/>
+      <c r="K37" s="12"/>
+      <c r="L37" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>48</v>
       </c>
@@ -1620,114 +1947,152 @@
       <c r="F38" s="15"/>
       <c r="G38" s="15"/>
       <c r="H38" s="15"/>
-      <c r="I38" s="10"/>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I38" s="15"/>
+      <c r="J38" s="15"/>
+      <c r="K38" s="15"/>
+      <c r="L38" s="10"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>49</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="C39" s="11"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="12"/>
+      <c r="C39" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="D39" s="11"/>
+      <c r="E39" s="11"/>
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
       <c r="H39" s="12"/>
-      <c r="I39" s="9"/>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I39" s="12"/>
+      <c r="J39" s="12"/>
+      <c r="K39" s="12"/>
+      <c r="L39" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="40" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>53</v>
       </c>
       <c r="B40" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="C40" s="14"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
+      <c r="C40" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
       <c r="F40" s="13"/>
       <c r="G40" s="13"/>
-      <c r="H40" s="12"/>
-      <c r="I40" s="9"/>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H40" s="13"/>
+      <c r="I40" s="13"/>
+      <c r="J40" s="12"/>
+      <c r="K40" s="12"/>
+      <c r="L40" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="41" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>50</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="C41" s="14"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="13"/>
+      <c r="C41" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14"/>
       <c r="F41" s="13"/>
       <c r="G41" s="13"/>
-      <c r="H41" s="12"/>
-      <c r="I41" s="9"/>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H41" s="13"/>
+      <c r="I41" s="13"/>
+      <c r="J41" s="12"/>
+      <c r="K41" s="12"/>
+      <c r="L41" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="42" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>51</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="C42" s="14"/>
-      <c r="D42" s="13"/>
-      <c r="E42" s="13"/>
+      <c r="C42" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
       <c r="F42" s="13"/>
       <c r="G42" s="13"/>
-      <c r="H42" s="12"/>
-      <c r="I42" s="9"/>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H42" s="13"/>
+      <c r="I42" s="13"/>
+      <c r="J42" s="12"/>
+      <c r="K42" s="12"/>
+      <c r="L42" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>55</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="C43" s="14"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
+      <c r="C43" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
       <c r="F43" s="13"/>
       <c r="G43" s="13"/>
-      <c r="H43" s="12"/>
-      <c r="I43" s="9"/>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H43" s="13"/>
+      <c r="I43" s="13"/>
+      <c r="J43" s="12"/>
+      <c r="K43" s="12"/>
+      <c r="L43" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="44" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>54</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C44" s="14"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
+      <c r="C44" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
       <c r="F44" s="13"/>
       <c r="G44" s="13"/>
-      <c r="H44" s="12"/>
-      <c r="I44" s="9"/>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H44" s="13"/>
+      <c r="I44" s="13"/>
+      <c r="J44" s="12"/>
+      <c r="K44" s="12"/>
+      <c r="L44" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="45" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
         <v>56</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="C45" s="14"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="13"/>
+      <c r="C45" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="D45" s="14"/>
+      <c r="E45" s="14"/>
       <c r="F45" s="13"/>
       <c r="G45" s="13"/>
-      <c r="H45" s="12"/>
-      <c r="I45" s="9"/>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H45" s="13"/>
+      <c r="I45" s="13"/>
+      <c r="J45" s="12"/>
+      <c r="K45" s="12"/>
+      <c r="L45" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="46" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>92</v>
       </c>
@@ -1738,127 +2103,172 @@
       <c r="F46" s="15"/>
       <c r="G46" s="15"/>
       <c r="H46" s="15"/>
-      <c r="I46" s="10"/>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I46" s="15"/>
+      <c r="J46" s="15"/>
+      <c r="K46" s="15"/>
+      <c r="L46" s="10"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="47" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
         <v>93</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="C47" s="11"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
+      <c r="C47" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="D47" s="11"/>
+      <c r="E47" s="11"/>
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
       <c r="H47" s="12"/>
-      <c r="I47" s="9" t="s">
+      <c r="I47" s="12"/>
+      <c r="J47" s="12"/>
+      <c r="K47" s="12"/>
+      <c r="L47" s="9" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="48" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
         <v>94</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="C48" s="14"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
+      <c r="C48" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="D48" s="14"/>
+      <c r="E48" s="14"/>
       <c r="F48" s="13"/>
       <c r="G48" s="13"/>
-      <c r="H48" s="12"/>
-      <c r="I48" s="9"/>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H48" s="13"/>
+      <c r="I48" s="13"/>
+      <c r="J48" s="12"/>
+      <c r="K48" s="12"/>
+      <c r="L48" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="49" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>96</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="C49" s="14"/>
-      <c r="D49" s="13"/>
-      <c r="E49" s="13"/>
+      <c r="C49" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="D49" s="14"/>
+      <c r="E49" s="14"/>
       <c r="F49" s="13"/>
       <c r="G49" s="13"/>
-      <c r="H49" s="12"/>
-      <c r="I49" s="9"/>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H49" s="13"/>
+      <c r="I49" s="13"/>
+      <c r="J49" s="12"/>
+      <c r="K49" s="12"/>
+      <c r="L49" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="50" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>97</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="C50" s="14"/>
-      <c r="D50" s="13"/>
-      <c r="E50" s="13"/>
+      <c r="C50" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D50" s="14"/>
+      <c r="E50" s="14"/>
       <c r="F50" s="13"/>
       <c r="G50" s="13"/>
-      <c r="H50" s="12"/>
-      <c r="I50" s="9"/>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H50" s="13"/>
+      <c r="I50" s="13"/>
+      <c r="J50" s="12"/>
+      <c r="K50" s="12"/>
+      <c r="L50" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="51" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>98</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="C51" s="14"/>
-      <c r="D51" s="13"/>
-      <c r="E51" s="13"/>
+      <c r="C51" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D51" s="14"/>
+      <c r="E51" s="14"/>
       <c r="F51" s="13"/>
       <c r="G51" s="13"/>
-      <c r="H51" s="12"/>
-      <c r="I51" s="9"/>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H51" s="13"/>
+      <c r="I51" s="13"/>
+      <c r="J51" s="12"/>
+      <c r="K51" s="12"/>
+      <c r="L51" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="52" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
         <v>99</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="C52" s="14"/>
-      <c r="D52" s="13"/>
-      <c r="E52" s="13"/>
+      <c r="C52" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="D52" s="14"/>
+      <c r="E52" s="14"/>
       <c r="F52" s="13"/>
       <c r="G52" s="13"/>
-      <c r="H52" s="12"/>
-      <c r="I52" s="9"/>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H52" s="13"/>
+      <c r="I52" s="13"/>
+      <c r="J52" s="12"/>
+      <c r="K52" s="12"/>
+      <c r="L52" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="53" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
         <v>110</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="C53" s="14"/>
-      <c r="D53" s="13"/>
-      <c r="E53" s="13"/>
+      <c r="C53" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="D53" s="14"/>
+      <c r="E53" s="14"/>
       <c r="F53" s="13"/>
       <c r="G53" s="13"/>
-      <c r="H53" s="12"/>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H53" s="13"/>
+      <c r="I53" s="13"/>
+      <c r="J53" s="12"/>
+      <c r="K53" s="16"/>
+      <c r="L53" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="54" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
         <v>113</v>
       </c>
       <c r="B54" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="C54" s="14"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="13"/>
+      <c r="C54" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="D54" s="14"/>
+      <c r="E54" s="14"/>
       <c r="F54" s="13"/>
       <c r="G54" s="13"/>
-      <c r="H54" s="12"/>
+      <c r="H54" s="13"/>
+      <c r="I54" s="13"/>
+      <c r="J54" s="12"/>
+      <c r="K54" s="16"/>
+      <c r="L54" s="0"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1867,6 +2277,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100841FCFF63B2DEE4FAB3ABDCB2B58E191" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6537ae6c172b48d8001feb3057ef3193">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f38bd768-81b4-450c-b73d-1a8fa3ba2722" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e79d1da23033c2d9c1658a7b9c3763cb" ns2:_="">
     <xsd:import namespace="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
@@ -2038,26 +2467,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5DB6742-085C-4A8F-8C68-EE166C6FD496}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0D3B35F-2651-4930-8D88-666C35501CF8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2073,22 +2501,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5DB6742-085C-4A8F-8C68-EE166C6FD496}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added progress bar, cleaned up code, and improved plot display
</commit_message>
<xml_diff>
--- a/Sizing/concepts_tabulations.xlsx
+++ b/Sizing/concepts_tabulations.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12514195-5942-4AE4-97F2-7ED29CB638FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D84227-C30F-4AE0-83B7-513683F019B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Concepts" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" fullCalcOnLoad="true" iterate="true"/>
+  <calcPr calcId="191029" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="374" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="171">
   <si>
     <t>Deliverable</t>
   </si>
@@ -209,9 +209,6 @@
     <t>Wing Area [m2]</t>
   </si>
   <si>
-    <t>F/A-18E</t>
-  </si>
-  <si>
     <t>17.54</t>
   </si>
   <si>
@@ -356,15 +353,6 @@
     <t>23900.0861</t>
   </si>
   <si>
-    <t>732.9451</t>
-  </si>
-  <si>
-    <t>505.5753</t>
-  </si>
-  <si>
-    <t>911.1361</t>
-  </si>
-  <si>
     <t>6.6602</t>
   </si>
   <si>
@@ -374,9 +362,6 @@
     <t>Max Sustained Turn Rate [deg/s]</t>
   </si>
   <si>
-    <t>0.062744</t>
-  </si>
-  <si>
     <t>Landing SEROC</t>
   </si>
   <si>
@@ -413,30 +398,9 @@
     <t>-0.1089</t>
   </si>
   <si>
-    <t>28.4223</t>
-  </si>
-  <si>
-    <t>16.5467</t>
-  </si>
-  <si>
     <t>Uses 1.3x stall (this is at MTOW)</t>
   </si>
   <si>
-    <t>145.3531</t>
-  </si>
-  <si>
-    <t>1298.9508</t>
-  </si>
-  <si>
-    <t>0.0024352</t>
-  </si>
-  <si>
-    <t>-1.5979</t>
-  </si>
-  <si>
-    <t>F/A-18E_Sized</t>
-  </si>
-  <si>
     <t>F-16</t>
   </si>
   <si>
@@ -449,9 +413,6 @@
     <t>911.0097</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
     <t>Temp</t>
   </si>
   <si>
@@ -464,54 +425,15 @@
     <t>1.6675</t>
   </si>
   <si>
-    <t>98.0516</t>
-  </si>
-  <si>
     <t>63.0246</t>
   </si>
   <si>
     <t>138.2653</t>
   </si>
   <si>
-    <t>1304.2817</t>
-  </si>
-  <si>
-    <t>40.6897</t>
-  </si>
-  <si>
-    <t>26.2351</t>
-  </si>
-  <si>
-    <t>2288.2981</t>
-  </si>
-  <si>
-    <t>426.048</t>
-  </si>
-  <si>
-    <t>1115.6452</t>
-  </si>
-  <si>
-    <t>763.9478</t>
-  </si>
-  <si>
-    <t>1309.7927</t>
-  </si>
-  <si>
-    <t>5624.6918</t>
-  </si>
-  <si>
-    <t>5.0621</t>
-  </si>
-  <si>
-    <t>2733.3813</t>
-  </si>
-  <si>
     <t>0.72081</t>
   </si>
   <si>
-    <t>10.1342</t>
-  </si>
-  <si>
     <t>27600.4439</t>
   </si>
   <si>
@@ -536,32 +458,104 @@
     <t>93.4938</t>
   </si>
   <si>
-    <t>-0.00018341</t>
-  </si>
-  <si>
-    <t>-0.32378</t>
-  </si>
-  <si>
     <t>-0.18621</t>
   </si>
   <si>
-    <t>-0.0014064</t>
-  </si>
-  <si>
     <t>-0.36166</t>
   </si>
   <si>
     <t>-0.7396</t>
   </si>
   <si>
-    <t>-1.6086</t>
+    <t>170.5489</t>
+  </si>
+  <si>
+    <t>2480.9254</t>
+  </si>
+  <si>
+    <t>24.4519</t>
+  </si>
+  <si>
+    <t>16.167</t>
+  </si>
+  <si>
+    <t>0.1762</t>
+  </si>
+  <si>
+    <t>-0.034213</t>
+  </si>
+  <si>
+    <t>-3.9619</t>
+  </si>
+  <si>
+    <t>111.2554</t>
+  </si>
+  <si>
+    <t>1991.6565</t>
+  </si>
+  <si>
+    <t>36.0863</t>
+  </si>
+  <si>
+    <t>25.9986</t>
+  </si>
+  <si>
+    <t>2288.6897</t>
+  </si>
+  <si>
+    <t>426.0548</t>
+  </si>
+  <si>
+    <t>1116.1852</t>
+  </si>
+  <si>
+    <t>763.9237</t>
+  </si>
+  <si>
+    <t>1310.6232</t>
+  </si>
+  <si>
+    <t>5617.6582</t>
+  </si>
+  <si>
+    <t>5.7256</t>
+  </si>
+  <si>
+    <t>2733.3788</t>
+  </si>
+  <si>
+    <t>10.1343</t>
+  </si>
+  <si>
+    <t>-0.027845</t>
+  </si>
+  <si>
+    <t>-0.00020745</t>
+  </si>
+  <si>
+    <t>-0.23272</t>
+  </si>
+  <si>
+    <t>-0.045178</t>
+  </si>
+  <si>
+    <t>-0.0014053</t>
+  </si>
+  <si>
+    <t>-2.9833</t>
+  </si>
+  <si>
+    <t>FA-18E</t>
+  </si>
+  <si>
+    <t>FA-18E Sized</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -595,13 +589,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519242"/>
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407453"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -612,7 +606,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -733,62 +727,60 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -807,7 +799,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -958,7 +950,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="true">
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -982,9 +974,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="true">
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1008,7 +1000,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1043,7 +1035,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -1061,7 +1053,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="true">
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1086,7 +1078,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -1122,36 +1114,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
   <dimension ref="A1:L54"/>
-  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.796875" customWidth="true"/>
-    <col min="2" max="2" width="10.5" customWidth="true"/>
-    <col min="3" max="3" width="13.5" customWidth="true"/>
-    <col min="4" max="4" width="4.69921875" customWidth="true"/>
-    <col min="6" max="6" width="9.796875" customWidth="true"/>
-    <col min="12" max="12" width="106.796875" customWidth="true"/>
-    <col min="5" max="5" width="4.69921875" customWidth="true"/>
-    <col min="7" max="7" width="9.796875" customWidth="true"/>
-    <col min="8" max="8" width="9.796875" customWidth="true"/>
-    <col min="9" max="9" width="9.796875" customWidth="true"/>
-    <col min="10" max="10" width="9.796875" customWidth="true"/>
-    <col min="11" max="11" width="6" customWidth="true"/>
+    <col min="1" max="1" width="38.77734375" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" customWidth="1"/>
+    <col min="3" max="3" width="13.44140625" customWidth="1"/>
+    <col min="4" max="5" width="4.6640625" customWidth="1"/>
+    <col min="6" max="10" width="9.77734375" customWidth="1"/>
+    <col min="11" max="11" width="6" customWidth="1"/>
+    <col min="12" max="12" width="106.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" ht="15" thickBot="true" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>57</v>
+        <v>169</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>132</v>
+        <v>170</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>8</v>
@@ -1160,7 +1147,7 @@
         <v>1</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>2</v>
@@ -1172,13 +1159,13 @@
         <v>4</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="L1" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1194,15 +1181,15 @@
       <c r="K2" s="3"/>
       <c r="L2" s="7"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="D3" s="11"/>
       <c r="E3" s="11"/>
@@ -1213,18 +1200,18 @@
       <c r="J3" s="13"/>
       <c r="K3" s="13"/>
       <c r="L3" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
-        <v>84</v>
-      </c>
       <c r="B4" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="11"/>
@@ -1235,18 +1222,18 @@
       <c r="J4" s="13"/>
       <c r="K4" s="13"/>
       <c r="L4" s="8" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D5" s="11"/>
       <c r="E5" s="11"/>
@@ -1260,15 +1247,15 @@
         <v>32</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>34</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D6" s="11"/>
       <c r="E6" s="11"/>
@@ -1282,15 +1269,15 @@
         <v>32</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>31</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="D7" s="11"/>
       <c r="E7" s="11"/>
@@ -1304,15 +1291,15 @@
         <v>35</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="11"/>
@@ -1323,18 +1310,18 @@
       <c r="J8" s="13"/>
       <c r="K8" s="13"/>
       <c r="L8" s="8" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>36</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="11"/>
@@ -1346,15 +1333,15 @@
       <c r="K9" s="13"/>
       <c r="L9" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>37</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="11"/>
@@ -1366,15 +1353,15 @@
       <c r="K10" s="13"/>
       <c r="L10" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
@@ -1386,15 +1373,15 @@
       <c r="K11" s="13"/>
       <c r="L11" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>38</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="11"/>
@@ -1406,15 +1393,15 @@
       <c r="K12" s="13"/>
       <c r="L12" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>126</v>
+        <v>146</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="11"/>
@@ -1426,15 +1413,15 @@
       <c r="K13" s="13"/>
       <c r="L13" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="D14" s="11"/>
       <c r="E14" s="11"/>
@@ -1448,15 +1435,15 @@
         <v>39</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="11"/>
@@ -1470,15 +1457,15 @@
         <v>40</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>43</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="D16" s="11"/>
       <c r="E16" s="11"/>
@@ -1490,15 +1477,15 @@
       <c r="K16" s="12"/>
       <c r="L16" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>44</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
@@ -1510,15 +1497,15 @@
       <c r="K17" s="12"/>
       <c r="L17" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>45</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D18" s="11"/>
       <c r="E18" s="11"/>
@@ -1530,15 +1517,15 @@
       <c r="K18" s="12"/>
       <c r="L18" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>41</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
@@ -1550,15 +1537,15 @@
       <c r="K19" s="12"/>
       <c r="L19" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>42</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
@@ -1570,15 +1557,15 @@
       <c r="K20" s="12"/>
       <c r="L20" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>46</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="D21" s="11"/>
       <c r="E21" s="11"/>
@@ -1592,15 +1579,15 @@
         <v>47</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>156</v>
+        <v>131</v>
       </c>
       <c r="D22" s="11"/>
       <c r="E22" s="11"/>
@@ -1614,15 +1601,15 @@
         <v>47</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>6</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="D23" s="11"/>
       <c r="E23" s="11"/>
@@ -1636,7 +1623,7 @@
         <v>47</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>24</v>
       </c>
@@ -1652,20 +1639,20 @@
       <c r="K24" s="15"/>
       <c r="L24" s="10"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D25" s="11"/>
       <c r="E25" s="11"/>
       <c r="F25" s="12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="12"/>
@@ -1676,15 +1663,15 @@
         <v>10</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D26" s="11"/>
       <c r="E26" s="11"/>
@@ -1698,15 +1685,15 @@
         <v>12</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>13</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D27" s="11"/>
       <c r="E27" s="11"/>
@@ -1720,20 +1707,20 @@
         <v>14</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>15</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D28" s="11"/>
       <c r="E28" s="11"/>
       <c r="F28" s="12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G28" s="12"/>
       <c r="H28" s="12"/>
@@ -1744,15 +1731,15 @@
         <v>16</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>17</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>158</v>
+        <v>132</v>
       </c>
       <c r="D29" s="11"/>
       <c r="E29" s="11"/>
@@ -1766,15 +1753,15 @@
         <v>18</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D30" s="11"/>
       <c r="E30" s="11"/>
@@ -1788,15 +1775,15 @@
         <v>27</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>25</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>159</v>
+        <v>133</v>
       </c>
       <c r="D31" s="11"/>
       <c r="E31" s="11"/>
@@ -1808,15 +1795,15 @@
       <c r="K31" s="12"/>
       <c r="L31" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>19</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D32" s="11"/>
       <c r="E32" s="11"/>
@@ -1830,15 +1817,15 @@
         <v>20</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>21</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>160</v>
+        <v>134</v>
       </c>
       <c r="D33" s="11"/>
       <c r="E33" s="11"/>
@@ -1852,15 +1839,15 @@
         <v>22</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="D34" s="11"/>
       <c r="E34" s="11"/>
@@ -1872,15 +1859,15 @@
       <c r="K34" s="12"/>
       <c r="L34" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D35" s="11"/>
       <c r="E35" s="11"/>
@@ -1891,10 +1878,10 @@
       <c r="J35" s="12"/>
       <c r="K35" s="12"/>
       <c r="L35" s="9" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>28</v>
       </c>
@@ -1916,15 +1903,15 @@
         <v>30</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>52</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D37" s="11"/>
       <c r="E37" s="11"/>
@@ -1936,7 +1923,7 @@
       <c r="K37" s="12"/>
       <c r="L37" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>48</v>
       </c>
@@ -1952,15 +1939,15 @@
       <c r="K38" s="15"/>
       <c r="L38" s="10"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>49</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>162</v>
+        <v>136</v>
       </c>
       <c r="D39" s="11"/>
       <c r="E39" s="11"/>
@@ -1972,15 +1959,15 @@
       <c r="K39" s="12"/>
       <c r="L39" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="40" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>53</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>163</v>
+        <v>137</v>
       </c>
       <c r="D40" s="14"/>
       <c r="E40" s="14"/>
@@ -1992,15 +1979,15 @@
       <c r="K40" s="12"/>
       <c r="L40" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="41" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>50</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D41" s="14"/>
       <c r="E41" s="14"/>
@@ -2012,15 +1999,15 @@
       <c r="K41" s="12"/>
       <c r="L41" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="42" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>51</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D42" s="14"/>
       <c r="E42" s="14"/>
@@ -2032,15 +2019,15 @@
       <c r="K42" s="12"/>
       <c r="L42" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>55</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>164</v>
+        <v>138</v>
       </c>
       <c r="D43" s="14"/>
       <c r="E43" s="14"/>
@@ -2052,15 +2039,15 @@
       <c r="K43" s="12"/>
       <c r="L43" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="44" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>54</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>72</v>
+        <v>163</v>
       </c>
       <c r="D44" s="14"/>
       <c r="E44" s="14"/>
@@ -2072,15 +2059,15 @@
       <c r="K44" s="12"/>
       <c r="L44" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="45" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
         <v>56</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>165</v>
+        <v>139</v>
       </c>
       <c r="D45" s="14"/>
       <c r="E45" s="14"/>
@@ -2092,9 +2079,9 @@
       <c r="K45" s="12"/>
       <c r="L45" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="46" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B46" s="15"/>
       <c r="C46" s="15"/>
@@ -2108,15 +2095,15 @@
       <c r="K46" s="15"/>
       <c r="L46" s="10"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="47" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D47" s="11"/>
       <c r="E47" s="11"/>
@@ -2127,18 +2114,18 @@
       <c r="J47" s="12"/>
       <c r="K47" s="12"/>
       <c r="L47" s="9" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="48" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D48" s="14"/>
       <c r="E48" s="14"/>
@@ -2150,15 +2137,15 @@
       <c r="K48" s="12"/>
       <c r="L48" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="49" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>112</v>
+        <v>148</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>137</v>
+        <v>166</v>
       </c>
       <c r="D49" s="14"/>
       <c r="E49" s="14"/>
@@ -2170,15 +2157,15 @@
       <c r="K49" s="12"/>
       <c r="L49" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="50" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="D50" s="14"/>
       <c r="E50" s="14"/>
@@ -2190,15 +2177,15 @@
       <c r="K50" s="12"/>
       <c r="L50" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="51" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D51" s="14"/>
       <c r="E51" s="14"/>
@@ -2210,15 +2197,15 @@
       <c r="K51" s="12"/>
       <c r="L51" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="52" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>170</v>
+        <v>141</v>
       </c>
       <c r="D52" s="14"/>
       <c r="E52" s="14"/>
@@ -2230,15 +2217,15 @@
       <c r="K52" s="12"/>
       <c r="L52" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="53" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>171</v>
+        <v>142</v>
       </c>
       <c r="D53" s="14"/>
       <c r="E53" s="14"/>
@@ -2248,17 +2235,16 @@
       <c r="I53" s="13"/>
       <c r="J53" s="12"/>
       <c r="K53" s="16"/>
-      <c r="L53" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="54" x14ac:dyDescent="0.3">
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>131</v>
+        <v>149</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D54" s="14"/>
       <c r="E54" s="14"/>
@@ -2268,7 +2254,6 @@
       <c r="I54" s="13"/>
       <c r="J54" s="12"/>
       <c r="K54" s="16"/>
-      <c r="L54" s="0"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2277,25 +2262,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100841FCFF63B2DEE4FAB3ABDCB2B58E191" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6537ae6c172b48d8001feb3057ef3193">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f38bd768-81b4-450c-b73d-1a8fa3ba2722" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e79d1da23033c2d9c1658a7b9c3763cb" ns2:_="">
     <xsd:import namespace="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
@@ -2467,10 +2433,39 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0D3B35F-2651-4930-8D88-666C35501CF8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2486,19 +2481,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0D3B35F-2651-4930-8D88-666C35501CF8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Performance plots in another function. Adding notes to concept_control
</commit_message>
<xml_diff>
--- a/Sizing/concepts_tabulations.xlsx
+++ b/Sizing/concepts_tabulations.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D84227-C30F-4AE0-83B7-513683F019B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1321B93-04D9-4CA1-8592-7C23F99AA06B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
     <sheet name="Concepts" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="true" iterate="true"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="943" uniqueCount="224">
   <si>
     <t>Deliverable</t>
   </si>
@@ -549,13 +549,172 @@
   </si>
   <si>
     <t>FA-18E Sized</t>
+  </si>
+  <si>
+    <t>1.2345</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>2500</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>0.5</t>
+  </si>
+  <si>
+    <t>4.5</t>
+  </si>
+  <si>
+    <t>0.33333</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>29.0546</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>-0.015748</t>
+  </si>
+  <si>
+    <t>88.2746</t>
+  </si>
+  <si>
+    <t>111.3531</t>
+  </si>
+  <si>
+    <t>276.31</t>
+  </si>
+  <si>
+    <t>1.8286</t>
+  </si>
+  <si>
+    <t>149.3268</t>
+  </si>
+  <si>
+    <t>61.5607</t>
+  </si>
+  <si>
+    <t>168.1095</t>
+  </si>
+  <si>
+    <t>1122.685</t>
+  </si>
+  <si>
+    <t>24.7998</t>
+  </si>
+  <si>
+    <t>20.5136</t>
+  </si>
+  <si>
+    <t>2099.7648</t>
+  </si>
+  <si>
+    <t>351.725</t>
+  </si>
+  <si>
+    <t>1054.1178</t>
+  </si>
+  <si>
+    <t>791.8646</t>
+  </si>
+  <si>
+    <t>1221.1825</t>
+  </si>
+  <si>
+    <t>7414.0166</t>
+  </si>
+  <si>
+    <t>1243.0346</t>
+  </si>
+  <si>
+    <t>4817.0198</t>
+  </si>
+  <si>
+    <t>0.79668</t>
+  </si>
+  <si>
+    <t>8.0252</t>
+  </si>
+  <si>
+    <t>36000</t>
+  </si>
+  <si>
+    <t>77969.4578</t>
+  </si>
+  <si>
+    <t>34331.4578</t>
+  </si>
+  <si>
+    <t>-0.034529</t>
+  </si>
+  <si>
+    <t>0.02984</t>
+  </si>
+  <si>
+    <t>-0.16164</t>
+  </si>
+  <si>
+    <t>-0.25473</t>
+  </si>
+  <si>
+    <t>-0.13367</t>
+  </si>
+  <si>
+    <t>-0.4544</t>
+  </si>
+  <si>
+    <t>-1.2454</t>
+  </si>
+  <si>
+    <t>1.6892</t>
+  </si>
+  <si>
+    <t>53.3798</t>
+  </si>
+  <si>
+    <t>93.1606</t>
+  </si>
+  <si>
+    <t>16.7378</t>
+  </si>
+  <si>
+    <t>7838.9933</t>
+  </si>
+  <si>
+    <t>1260.8647</t>
+  </si>
+  <si>
+    <t>0.53112</t>
+  </si>
+  <si>
+    <t>-0.035024</t>
+  </si>
+  <si>
+    <t>-0.059402</t>
+  </si>
+  <si>
+    <t>-0.13837</t>
+  </si>
+  <si>
+    <t>-0.06663</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -589,13 +748,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
+        <fgColor theme="4" tint="0.39997558519242"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="0" tint="-0.14999847407453"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -720,67 +879,59 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -799,7 +950,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -950,7 +1101,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -974,9 +1125,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1000,7 +1151,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1035,7 +1186,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -1053,7 +1204,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1078,7 +1229,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -1114,20 +1265,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
   <dimension ref="A1:L54"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.77734375" customWidth="1"/>
-    <col min="2" max="2" width="10.44140625" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" customWidth="1"/>
-    <col min="4" max="5" width="4.6640625" customWidth="1"/>
-    <col min="6" max="10" width="9.77734375" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="106.77734375" customWidth="1"/>
+    <col min="1" max="1" width="38.796875" customWidth="true"/>
+    <col min="2" max="2" width="10.5" customWidth="true"/>
+    <col min="3" max="3" width="12.5" customWidth="true"/>
+    <col min="4" max="4" width="4.69921875" customWidth="true"/>
+    <col min="6" max="6" width="9.796875" customWidth="true"/>
+    <col min="11" max="11" width="10.5" customWidth="true"/>
+    <col min="12" max="12" width="106.796875" customWidth="true"/>
+    <col min="5" max="5" width="4.69921875" customWidth="true"/>
+    <col min="7" max="7" width="9.796875" customWidth="true"/>
+    <col min="8" max="8" width="9.796875" customWidth="true"/>
+    <col min="9" max="9" width="9.796875" customWidth="true"/>
+    <col min="10" max="10" width="9.796875" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" ht="15" thickBot="true" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1165,7 +1321,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1181,7 +1337,7 @@
       <c r="K2" s="3"/>
       <c r="L2" s="7"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>81</v>
       </c>
@@ -1198,12 +1354,14 @@
       <c r="H3" s="12"/>
       <c r="I3" s="12"/>
       <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
+      <c r="K3" s="13" t="s">
+        <v>183</v>
+      </c>
       <c r="L3" s="8" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>83</v>
       </c>
@@ -1220,12 +1378,14 @@
       <c r="H4" s="12"/>
       <c r="I4" s="12"/>
       <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
+      <c r="K4" s="13" t="s">
+        <v>171</v>
+      </c>
       <c r="L4" s="8" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
@@ -1242,12 +1402,14 @@
       <c r="H5" s="12"/>
       <c r="I5" s="12"/>
       <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
+      <c r="K5" s="13" t="s">
+        <v>79</v>
+      </c>
       <c r="L5" s="8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>34</v>
       </c>
@@ -1264,12 +1426,14 @@
       <c r="H6" s="12"/>
       <c r="I6" s="12"/>
       <c r="J6" s="13"/>
-      <c r="K6" s="13"/>
+      <c r="K6" s="13" t="s">
+        <v>80</v>
+      </c>
       <c r="L6" s="8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>31</v>
       </c>
@@ -1286,12 +1450,14 @@
       <c r="H7" s="12"/>
       <c r="I7" s="12"/>
       <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
+      <c r="K7" s="13" t="s">
+        <v>213</v>
+      </c>
       <c r="L7" s="8" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>87</v>
       </c>
@@ -1308,12 +1474,14 @@
       <c r="H8" s="12"/>
       <c r="I8" s="12"/>
       <c r="J8" s="13"/>
-      <c r="K8" s="13"/>
+      <c r="K8" s="13" t="s">
+        <v>187</v>
+      </c>
       <c r="L8" s="8" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>36</v>
       </c>
@@ -1330,10 +1498,12 @@
       <c r="H9" s="12"/>
       <c r="I9" s="12"/>
       <c r="J9" s="13"/>
-      <c r="K9" s="13"/>
+      <c r="K9" s="13" t="s">
+        <v>214</v>
+      </c>
       <c r="L9" s="8"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>37</v>
       </c>
@@ -1350,10 +1520,12 @@
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
       <c r="J10" s="13"/>
-      <c r="K10" s="13"/>
+      <c r="K10" s="13" t="s">
+        <v>215</v>
+      </c>
       <c r="L10" s="8"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>109</v>
       </c>
@@ -1370,10 +1542,12 @@
       <c r="H11" s="12"/>
       <c r="I11" s="12"/>
       <c r="J11" s="13"/>
-      <c r="K11" s="13"/>
+      <c r="K11" s="13" t="s">
+        <v>190</v>
+      </c>
       <c r="L11" s="8"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>38</v>
       </c>
@@ -1390,10 +1564,12 @@
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
       <c r="J12" s="13"/>
-      <c r="K12" s="13"/>
+      <c r="K12" s="13" t="s">
+        <v>191</v>
+      </c>
       <c r="L12" s="8"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>107</v>
       </c>
@@ -1410,10 +1586,12 @@
       <c r="H13" s="12"/>
       <c r="I13" s="12"/>
       <c r="J13" s="13"/>
-      <c r="K13" s="13"/>
+      <c r="K13" s="13" t="s">
+        <v>216</v>
+      </c>
       <c r="L13" s="8"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>77</v>
       </c>
@@ -1430,12 +1608,14 @@
       <c r="H14" s="12"/>
       <c r="I14" s="12"/>
       <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
+      <c r="K14" s="12" t="s">
+        <v>193</v>
+      </c>
       <c r="L14" s="9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>78</v>
       </c>
@@ -1452,12 +1632,14 @@
       <c r="H15" s="12"/>
       <c r="I15" s="12"/>
       <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
+      <c r="K15" s="12" t="s">
+        <v>194</v>
+      </c>
       <c r="L15" s="9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>43</v>
       </c>
@@ -1474,10 +1656,12 @@
       <c r="H16" s="12"/>
       <c r="I16" s="12"/>
       <c r="J16" s="12"/>
-      <c r="K16" s="12"/>
+      <c r="K16" s="12" t="s">
+        <v>195</v>
+      </c>
       <c r="L16" s="9"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>44</v>
       </c>
@@ -1494,10 +1678,12 @@
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
       <c r="J17" s="12"/>
-      <c r="K17" s="12"/>
+      <c r="K17" s="12" t="s">
+        <v>196</v>
+      </c>
       <c r="L17" s="9"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>45</v>
       </c>
@@ -1514,10 +1700,12 @@
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
       <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
+      <c r="K18" s="12" t="s">
+        <v>197</v>
+      </c>
       <c r="L18" s="9"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>41</v>
       </c>
@@ -1534,10 +1722,12 @@
       <c r="H19" s="12"/>
       <c r="I19" s="12"/>
       <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
+      <c r="K19" s="12" t="s">
+        <v>217</v>
+      </c>
       <c r="L19" s="9"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>42</v>
       </c>
@@ -1554,10 +1744,12 @@
       <c r="H20" s="12"/>
       <c r="I20" s="12"/>
       <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
+      <c r="K20" s="12" t="s">
+        <v>218</v>
+      </c>
       <c r="L20" s="9"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>46</v>
       </c>
@@ -1574,12 +1766,14 @@
       <c r="H21" s="12"/>
       <c r="I21" s="12"/>
       <c r="J21" s="12"/>
-      <c r="K21" s="12"/>
+      <c r="K21" s="12" t="s">
+        <v>200</v>
+      </c>
       <c r="L21" s="9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>76</v>
       </c>
@@ -1596,12 +1790,14 @@
       <c r="H22" s="12"/>
       <c r="I22" s="12"/>
       <c r="J22" s="12"/>
-      <c r="K22" s="12"/>
+      <c r="K22" s="12" t="s">
+        <v>219</v>
+      </c>
       <c r="L22" s="9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>6</v>
       </c>
@@ -1618,12 +1814,14 @@
       <c r="H23" s="12"/>
       <c r="I23" s="12"/>
       <c r="J23" s="12"/>
-      <c r="K23" s="12"/>
+      <c r="K23" s="12" t="s">
+        <v>202</v>
+      </c>
       <c r="L23" s="9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>24</v>
       </c>
@@ -1639,7 +1837,7 @@
       <c r="K24" s="15"/>
       <c r="L24" s="10"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>9</v>
       </c>
@@ -1658,12 +1856,14 @@
       <c r="H25" s="12"/>
       <c r="I25" s="12"/>
       <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
+      <c r="K25" s="12" t="s">
+        <v>174</v>
+      </c>
       <c r="L25" s="9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>11</v>
       </c>
@@ -1680,12 +1880,14 @@
       <c r="H26" s="12"/>
       <c r="I26" s="12"/>
       <c r="J26" s="12"/>
-      <c r="K26" s="12"/>
+      <c r="K26" s="12" t="s">
+        <v>67</v>
+      </c>
       <c r="L26" s="9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>13</v>
       </c>
@@ -1702,12 +1904,14 @@
       <c r="H27" s="12"/>
       <c r="I27" s="12"/>
       <c r="J27" s="12"/>
-      <c r="K27" s="12"/>
+      <c r="K27" s="12" t="s">
+        <v>172</v>
+      </c>
       <c r="L27" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>15</v>
       </c>
@@ -1726,12 +1930,14 @@
       <c r="H28" s="12"/>
       <c r="I28" s="12"/>
       <c r="J28" s="12"/>
-      <c r="K28" s="12"/>
+      <c r="K28" s="12" t="s">
+        <v>60</v>
+      </c>
       <c r="L28" s="9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>17</v>
       </c>
@@ -1748,12 +1954,14 @@
       <c r="H29" s="12"/>
       <c r="I29" s="12"/>
       <c r="J29" s="12"/>
-      <c r="K29" s="12"/>
+      <c r="K29" s="12" t="s">
+        <v>203</v>
+      </c>
       <c r="L29" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>26</v>
       </c>
@@ -1770,12 +1978,14 @@
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
       <c r="J30" s="12"/>
-      <c r="K30" s="12"/>
+      <c r="K30" s="12" t="s">
+        <v>173</v>
+      </c>
       <c r="L30" s="9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>25</v>
       </c>
@@ -1792,10 +2002,12 @@
       <c r="H31" s="12"/>
       <c r="I31" s="12"/>
       <c r="J31" s="12"/>
-      <c r="K31" s="12"/>
+      <c r="K31" s="12" t="s">
+        <v>174</v>
+      </c>
       <c r="L31" s="9"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>19</v>
       </c>
@@ -1812,12 +2024,14 @@
       <c r="H32" s="12"/>
       <c r="I32" s="12"/>
       <c r="J32" s="12"/>
-      <c r="K32" s="12"/>
+      <c r="K32" s="12" t="s">
+        <v>175</v>
+      </c>
       <c r="L32" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>21</v>
       </c>
@@ -1834,12 +2048,14 @@
       <c r="H33" s="12"/>
       <c r="I33" s="12"/>
       <c r="J33" s="12"/>
-      <c r="K33" s="12"/>
+      <c r="K33" s="12" t="s">
+        <v>172</v>
+      </c>
       <c r="L33" s="9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>23</v>
       </c>
@@ -1856,10 +2072,12 @@
       <c r="H34" s="12"/>
       <c r="I34" s="12"/>
       <c r="J34" s="12"/>
-      <c r="K34" s="12"/>
+      <c r="K34" s="12" t="s">
+        <v>67</v>
+      </c>
       <c r="L34" s="9"/>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>85</v>
       </c>
@@ -1876,12 +2094,14 @@
       <c r="H35" s="12"/>
       <c r="I35" s="12"/>
       <c r="J35" s="12"/>
-      <c r="K35" s="12"/>
+      <c r="K35" s="12" t="s">
+        <v>176</v>
+      </c>
       <c r="L35" s="9" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>28</v>
       </c>
@@ -1898,12 +2118,14 @@
       <c r="H36" s="12"/>
       <c r="I36" s="12"/>
       <c r="J36" s="12"/>
-      <c r="K36" s="12"/>
+      <c r="K36" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="L36" s="9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>52</v>
       </c>
@@ -1920,10 +2142,12 @@
       <c r="H37" s="12"/>
       <c r="I37" s="12"/>
       <c r="J37" s="12"/>
-      <c r="K37" s="12"/>
+      <c r="K37" s="12" t="s">
+        <v>67</v>
+      </c>
       <c r="L37" s="9"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>48</v>
       </c>
@@ -1939,7 +2163,7 @@
       <c r="K38" s="15"/>
       <c r="L38" s="10"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>49</v>
       </c>
@@ -1956,10 +2180,12 @@
       <c r="H39" s="12"/>
       <c r="I39" s="12"/>
       <c r="J39" s="12"/>
-      <c r="K39" s="12"/>
+      <c r="K39" s="12" t="s">
+        <v>204</v>
+      </c>
       <c r="L39" s="9"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="40" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>53</v>
       </c>
@@ -1976,10 +2202,12 @@
       <c r="H40" s="13"/>
       <c r="I40" s="13"/>
       <c r="J40" s="12"/>
-      <c r="K40" s="12"/>
+      <c r="K40" s="12" t="s">
+        <v>205</v>
+      </c>
       <c r="L40" s="9"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="41" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>50</v>
       </c>
@@ -1996,10 +2224,12 @@
       <c r="H41" s="13"/>
       <c r="I41" s="13"/>
       <c r="J41" s="12"/>
-      <c r="K41" s="12"/>
+      <c r="K41" s="12" t="s">
+        <v>177</v>
+      </c>
       <c r="L41" s="9"/>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="42" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>51</v>
       </c>
@@ -2016,10 +2246,12 @@
       <c r="H42" s="13"/>
       <c r="I42" s="13"/>
       <c r="J42" s="12"/>
-      <c r="K42" s="12"/>
+      <c r="K42" s="12" t="s">
+        <v>178</v>
+      </c>
       <c r="L42" s="9"/>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>55</v>
       </c>
@@ -2036,10 +2268,12 @@
       <c r="H43" s="13"/>
       <c r="I43" s="13"/>
       <c r="J43" s="12"/>
-      <c r="K43" s="12"/>
+      <c r="K43" s="12" t="s">
+        <v>179</v>
+      </c>
       <c r="L43" s="9"/>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="44" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>54</v>
       </c>
@@ -2056,10 +2290,12 @@
       <c r="H44" s="13"/>
       <c r="I44" s="13"/>
       <c r="J44" s="12"/>
-      <c r="K44" s="12"/>
+      <c r="K44" s="12" t="s">
+        <v>180</v>
+      </c>
       <c r="L44" s="9"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="45" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
         <v>56</v>
       </c>
@@ -2076,10 +2312,12 @@
       <c r="H45" s="13"/>
       <c r="I45" s="13"/>
       <c r="J45" s="12"/>
-      <c r="K45" s="12"/>
+      <c r="K45" s="12" t="s">
+        <v>181</v>
+      </c>
       <c r="L45" s="9"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="46" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>91</v>
       </c>
@@ -2095,7 +2333,7 @@
       <c r="K46" s="15"/>
       <c r="L46" s="10"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="47" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
         <v>92</v>
       </c>
@@ -2112,12 +2350,14 @@
       <c r="H47" s="12"/>
       <c r="I47" s="12"/>
       <c r="J47" s="12"/>
-      <c r="K47" s="12"/>
+      <c r="K47" s="12" t="s">
+        <v>220</v>
+      </c>
       <c r="L47" s="9" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="48" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
         <v>93</v>
       </c>
@@ -2134,10 +2374,12 @@
       <c r="H48" s="13"/>
       <c r="I48" s="13"/>
       <c r="J48" s="12"/>
-      <c r="K48" s="12"/>
+      <c r="K48" s="12" t="s">
+        <v>207</v>
+      </c>
       <c r="L48" s="9"/>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="49" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>95</v>
       </c>
@@ -2154,10 +2396,12 @@
       <c r="H49" s="13"/>
       <c r="I49" s="13"/>
       <c r="J49" s="12"/>
-      <c r="K49" s="12"/>
+      <c r="K49" s="12" t="s">
+        <v>221</v>
+      </c>
       <c r="L49" s="9"/>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="50" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>96</v>
       </c>
@@ -2174,10 +2418,12 @@
       <c r="H50" s="13"/>
       <c r="I50" s="13"/>
       <c r="J50" s="12"/>
-      <c r="K50" s="12"/>
+      <c r="K50" s="12" t="s">
+        <v>222</v>
+      </c>
       <c r="L50" s="9"/>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="51" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>97</v>
       </c>
@@ -2194,10 +2440,12 @@
       <c r="H51" s="13"/>
       <c r="I51" s="13"/>
       <c r="J51" s="12"/>
-      <c r="K51" s="12"/>
+      <c r="K51" s="12" t="s">
+        <v>182</v>
+      </c>
       <c r="L51" s="9"/>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="52" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
         <v>98</v>
       </c>
@@ -2214,10 +2462,12 @@
       <c r="H52" s="13"/>
       <c r="I52" s="13"/>
       <c r="J52" s="12"/>
-      <c r="K52" s="12"/>
+      <c r="K52" s="12" t="s">
+        <v>210</v>
+      </c>
       <c r="L52" s="9"/>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="53" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
         <v>106</v>
       </c>
@@ -2234,9 +2484,12 @@
       <c r="H53" s="13"/>
       <c r="I53" s="13"/>
       <c r="J53" s="12"/>
-      <c r="K53" s="16"/>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K53" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="L53" s="9"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="54" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
         <v>108</v>
       </c>
@@ -2253,7 +2506,10 @@
       <c r="H54" s="13"/>
       <c r="I54" s="13"/>
       <c r="J54" s="12"/>
-      <c r="K54" s="16"/>
+      <c r="K54" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="L54" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
changing how concept control reads in a file cause it was not working for me, old one still is there
</commit_message>
<xml_diff>
--- a/Sizing/concepts_tabulations.xlsx
+++ b/Sizing/concepts_tabulations.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\garim\OneDrive\Desktop\Air-Vehicle-Design\team10aiaa\Sizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1321B93-04D9-4CA1-8592-7C23F99AA06B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A3F43EA-941B-4E7B-816D-981693179B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872"/>
   </bookViews>
   <sheets>
     <sheet name="Concepts" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="943" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="563" uniqueCount="275">
   <si>
     <t>Deliverable</t>
   </si>
@@ -590,33 +590,15 @@
     <t>88.2746</t>
   </si>
   <si>
-    <t>111.3531</t>
-  </si>
-  <si>
-    <t>276.31</t>
-  </si>
-  <si>
-    <t>1.8286</t>
-  </si>
-  <si>
     <t>149.3268</t>
   </si>
   <si>
-    <t>61.5607</t>
-  </si>
-  <si>
-    <t>168.1095</t>
-  </si>
-  <si>
     <t>1122.685</t>
   </si>
   <si>
     <t>24.7998</t>
   </si>
   <si>
-    <t>20.5136</t>
-  </si>
-  <si>
     <t>2099.7648</t>
   </si>
   <si>
@@ -632,18 +614,9 @@
     <t>1221.1825</t>
   </si>
   <si>
-    <t>7414.0166</t>
-  </si>
-  <si>
-    <t>1243.0346</t>
-  </si>
-  <si>
     <t>4817.0198</t>
   </si>
   <si>
-    <t>0.79668</t>
-  </si>
-  <si>
     <t>8.0252</t>
   </si>
   <si>
@@ -656,24 +629,12 @@
     <t>34331.4578</t>
   </si>
   <si>
-    <t>-0.034529</t>
-  </si>
-  <si>
     <t>0.02984</t>
   </si>
   <si>
-    <t>-0.16164</t>
-  </si>
-  <si>
-    <t>-0.25473</t>
-  </si>
-  <si>
     <t>-0.13367</t>
   </si>
   <si>
-    <t>-0.4544</t>
-  </si>
-  <si>
     <t>-1.2454</t>
   </si>
   <si>
@@ -708,6 +669,198 @@
   </si>
   <si>
     <t>-0.06663</t>
+  </si>
+  <si>
+    <t>98.4214</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>2.46</t>
+  </si>
+  <si>
+    <t>35000</t>
+  </si>
+  <si>
+    <t>12.197</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>0.3</t>
+  </si>
+  <si>
+    <t>75485.2192</t>
+  </si>
+  <si>
+    <t>33347.2192</t>
+  </si>
+  <si>
+    <t>-0.33306</t>
+  </si>
+  <si>
+    <t>-0.16128</t>
+  </si>
+  <si>
+    <t>0.5486</t>
+  </si>
+  <si>
+    <t>1.0008</t>
+  </si>
+  <si>
+    <t>1.5491</t>
+  </si>
+  <si>
+    <t>189.6599</t>
+  </si>
+  <si>
+    <t>47.8233</t>
+  </si>
+  <si>
+    <t>95.2547</t>
+  </si>
+  <si>
+    <t>1113.83</t>
+  </si>
+  <si>
+    <t>22.5243</t>
+  </si>
+  <si>
+    <t>12.7772</t>
+  </si>
+  <si>
+    <t>1714.1537</t>
+  </si>
+  <si>
+    <t>264.3489</t>
+  </si>
+  <si>
+    <t>2416.4261</t>
+  </si>
+  <si>
+    <t>-3601.6363</t>
+  </si>
+  <si>
+    <t>8031.4817</t>
+  </si>
+  <si>
+    <t>6.1167</t>
+  </si>
+  <si>
+    <t>4.9304</t>
+  </si>
+  <si>
+    <t>1.925</t>
+  </si>
+  <si>
+    <t>3.5584</t>
+  </si>
+  <si>
+    <t>0.39044</t>
+  </si>
+  <si>
+    <t>3.4277</t>
+  </si>
+  <si>
+    <t>11.7174</t>
+  </si>
+  <si>
+    <t>41.8074</t>
+  </si>
+  <si>
+    <t>0.1029</t>
+  </si>
+  <si>
+    <t>0.308</t>
+  </si>
+  <si>
+    <t>0.047131</t>
+  </si>
+  <si>
+    <t>-0.13989</t>
+  </si>
+  <si>
+    <t>0.17097</t>
+  </si>
+  <si>
+    <t>-1.2277</t>
+  </si>
+  <si>
+    <t>F135</t>
+  </si>
+  <si>
+    <t>74.9155</t>
+  </si>
+  <si>
+    <t>190.7849</t>
+  </si>
+  <si>
+    <t>1.5694</t>
+  </si>
+  <si>
+    <t>189.6592</t>
+  </si>
+  <si>
+    <t>48.4973</t>
+  </si>
+  <si>
+    <t>100.5459</t>
+  </si>
+  <si>
+    <t>6752.4623</t>
+  </si>
+  <si>
+    <t>22.5244</t>
+  </si>
+  <si>
+    <t>13.0052</t>
+  </si>
+  <si>
+    <t>1714.2096</t>
+  </si>
+  <si>
+    <t>264.3495</t>
+  </si>
+  <si>
+    <t>2402.513</t>
+  </si>
+  <si>
+    <t>-3584.369</t>
+  </si>
+  <si>
+    <t>8031.4232</t>
+  </si>
+  <si>
+    <t>0.56819</t>
+  </si>
+  <si>
+    <t>0.39043</t>
+  </si>
+  <si>
+    <t>11.7169</t>
+  </si>
+  <si>
+    <t>41.8077</t>
+  </si>
+  <si>
+    <t>0.10241</t>
+  </si>
+  <si>
+    <t>0.30799</t>
+  </si>
+  <si>
+    <t>0.03261</t>
+  </si>
+  <si>
+    <t>-0.14926</t>
+  </si>
+  <si>
+    <t>0.15478</t>
+  </si>
+  <si>
+    <t>-12.5049</t>
   </si>
 </sst>
 </file>
@@ -1267,23 +1420,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
   <dimension ref="A1:L54"/>
-  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="38.796875" customWidth="true"/>
-    <col min="2" max="2" width="10.5" customWidth="true"/>
-    <col min="3" max="3" width="12.5" customWidth="true"/>
-    <col min="4" max="4" width="4.69921875" customWidth="true"/>
-    <col min="6" max="6" width="9.796875" customWidth="true"/>
-    <col min="11" max="11" width="10.5" customWidth="true"/>
-    <col min="12" max="12" width="106.796875" customWidth="true"/>
-    <col min="5" max="5" width="4.69921875" customWidth="true"/>
-    <col min="7" max="7" width="9.796875" customWidth="true"/>
-    <col min="8" max="8" width="9.796875" customWidth="true"/>
-    <col min="9" max="9" width="9.796875" customWidth="true"/>
-    <col min="10" max="10" width="9.796875" customWidth="true"/>
+    <col min="1" max="1" width="37.85546875" customWidth="true"/>
+    <col min="2" max="2" width="10.5703125" customWidth="true"/>
+    <col min="3" max="3" width="12.33203125" customWidth="true"/>
+    <col min="4" max="4" width="4.76171875" customWidth="true"/>
+    <col min="6" max="6" width="9.7109375" customWidth="true"/>
+    <col min="9" max="9" width="10.5703125" customWidth="true"/>
+    <col min="10" max="10" width="9.7109375" customWidth="true"/>
+    <col min="11" max="11" width="10.5703125" customWidth="true"/>
+    <col min="12" max="12" width="99.90234375" customWidth="true"/>
+    <col min="5" max="5" width="4.76171875" customWidth="true"/>
+    <col min="7" max="7" width="9.7109375" customWidth="true"/>
+    <col min="8" max="8" width="9.7109375" customWidth="true"/>
   </cols>
   <sheetData>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" ht="15" thickBot="true" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" ht="14.7" thickBot="true" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1321,7 +1474,7 @@
         <v>7</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1337,7 +1490,7 @@
       <c r="K2" s="3"/>
       <c r="L2" s="7"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="5" t="s">
         <v>81</v>
       </c>
@@ -1352,7 +1505,9 @@
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
+      <c r="I3" s="12" t="s">
+        <v>211</v>
+      </c>
       <c r="J3" s="13"/>
       <c r="K3" s="13" t="s">
         <v>183</v>
@@ -1361,7 +1516,7 @@
         <v>82</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5" t="s">
         <v>83</v>
       </c>
@@ -1376,7 +1531,9 @@
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
       <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
+      <c r="I4" s="12" t="s">
+        <v>223</v>
+      </c>
       <c r="J4" s="13"/>
       <c r="K4" s="13" t="s">
         <v>171</v>
@@ -1385,7 +1542,7 @@
         <v>84</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
@@ -1400,7 +1557,9 @@
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
       <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
+      <c r="I5" s="12" t="s">
+        <v>251</v>
+      </c>
       <c r="J5" s="13"/>
       <c r="K5" s="13" t="s">
         <v>79</v>
@@ -1409,7 +1568,7 @@
         <v>32</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="5" t="s">
         <v>34</v>
       </c>
@@ -1424,7 +1583,9 @@
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
+      <c r="I6" s="12" t="s">
+        <v>252</v>
+      </c>
       <c r="J6" s="13"/>
       <c r="K6" s="13" t="s">
         <v>80</v>
@@ -1433,7 +1594,7 @@
         <v>32</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="5" t="s">
         <v>31</v>
       </c>
@@ -1448,16 +1609,18 @@
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
       <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
+      <c r="I7" s="12" t="s">
+        <v>253</v>
+      </c>
       <c r="J7" s="13"/>
       <c r="K7" s="13" t="s">
-        <v>213</v>
+        <v>200</v>
       </c>
       <c r="L7" s="8" t="s">
         <v>35</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="5" t="s">
         <v>87</v>
       </c>
@@ -1472,16 +1635,18 @@
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
       <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
+      <c r="I8" s="12" t="s">
+        <v>254</v>
+      </c>
       <c r="J8" s="13"/>
       <c r="K8" s="13" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="L8" s="8" t="s">
         <v>120</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="5" t="s">
         <v>36</v>
       </c>
@@ -1496,14 +1661,16 @@
       <c r="F9" s="12"/>
       <c r="G9" s="12"/>
       <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
+      <c r="I9" s="12" t="s">
+        <v>255</v>
+      </c>
       <c r="J9" s="13"/>
       <c r="K9" s="13" t="s">
-        <v>214</v>
+        <v>201</v>
       </c>
       <c r="L9" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="5" t="s">
         <v>37</v>
       </c>
@@ -1518,14 +1685,16 @@
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
       <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
+      <c r="I10" s="12" t="s">
+        <v>256</v>
+      </c>
       <c r="J10" s="13"/>
       <c r="K10" s="13" t="s">
-        <v>215</v>
+        <v>202</v>
       </c>
       <c r="L10" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="5" t="s">
         <v>109</v>
       </c>
@@ -1540,14 +1709,16 @@
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
       <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
+      <c r="I11" s="12" t="s">
+        <v>257</v>
+      </c>
       <c r="J11" s="13"/>
       <c r="K11" s="13" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="L11" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="5" t="s">
         <v>38</v>
       </c>
@@ -1562,14 +1733,16 @@
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>
       <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
+      <c r="I12" s="12" t="s">
+        <v>258</v>
+      </c>
       <c r="J12" s="13"/>
       <c r="K12" s="13" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="L12" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="5" t="s">
         <v>107</v>
       </c>
@@ -1584,14 +1757,16 @@
       <c r="F13" s="12"/>
       <c r="G13" s="12"/>
       <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
+      <c r="I13" s="12" t="s">
+        <v>259</v>
+      </c>
       <c r="J13" s="13"/>
       <c r="K13" s="13" t="s">
-        <v>216</v>
+        <v>203</v>
       </c>
       <c r="L13" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="5" t="s">
         <v>77</v>
       </c>
@@ -1606,16 +1781,18 @@
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
       <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
+      <c r="I14" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="J14" s="12"/>
       <c r="K14" s="12" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="L14" s="9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="5" t="s">
         <v>78</v>
       </c>
@@ -1630,16 +1807,18 @@
       <c r="F15" s="12"/>
       <c r="G15" s="12"/>
       <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
+      <c r="I15" s="12" t="s">
+        <v>261</v>
+      </c>
       <c r="J15" s="12"/>
       <c r="K15" s="12" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="L15" s="9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="5" t="s">
         <v>43</v>
       </c>
@@ -1657,11 +1836,11 @@
       <c r="I16" s="12"/>
       <c r="J16" s="12"/>
       <c r="K16" s="12" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="L16" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="5" t="s">
         <v>44</v>
       </c>
@@ -1679,11 +1858,11 @@
       <c r="I17" s="12"/>
       <c r="J17" s="12"/>
       <c r="K17" s="12" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="L17" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="5" t="s">
         <v>45</v>
       </c>
@@ -1701,11 +1880,11 @@
       <c r="I18" s="12"/>
       <c r="J18" s="12"/>
       <c r="K18" s="12" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="L18" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="5" t="s">
         <v>41</v>
       </c>
@@ -1720,14 +1899,16 @@
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
+      <c r="I19" s="12" t="s">
+        <v>262</v>
+      </c>
       <c r="J19" s="12"/>
       <c r="K19" s="12" t="s">
-        <v>217</v>
+        <v>204</v>
       </c>
       <c r="L19" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="5" t="s">
         <v>42</v>
       </c>
@@ -1742,14 +1923,16 @@
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
       <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
+      <c r="I20" s="12" t="s">
+        <v>263</v>
+      </c>
       <c r="J20" s="12"/>
       <c r="K20" s="12" t="s">
-        <v>218</v>
+        <v>205</v>
       </c>
       <c r="L20" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="5" t="s">
         <v>46</v>
       </c>
@@ -1764,16 +1947,18 @@
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
       <c r="H21" s="12"/>
-      <c r="I21" s="12"/>
+      <c r="I21" s="12" t="s">
+        <v>264</v>
+      </c>
       <c r="J21" s="12"/>
       <c r="K21" s="12" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="L21" s="9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="5" t="s">
         <v>76</v>
       </c>
@@ -1788,16 +1973,18 @@
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
       <c r="H22" s="12"/>
-      <c r="I22" s="12"/>
+      <c r="I22" s="12" t="s">
+        <v>265</v>
+      </c>
       <c r="J22" s="12"/>
       <c r="K22" s="12" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="L22" s="9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="5" t="s">
         <v>6</v>
       </c>
@@ -1812,16 +1999,18 @@
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
       <c r="H23" s="12"/>
-      <c r="I23" s="12"/>
+      <c r="I23" s="12" t="s">
+        <v>236</v>
+      </c>
       <c r="J23" s="12"/>
       <c r="K23" s="12" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="L23" s="9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="4" t="s">
         <v>24</v>
       </c>
@@ -1837,7 +2026,7 @@
       <c r="K24" s="15"/>
       <c r="L24" s="10"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="5" t="s">
         <v>9</v>
       </c>
@@ -1854,7 +2043,9 @@
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="12"/>
-      <c r="I25" s="12"/>
+      <c r="I25" s="12" t="s">
+        <v>212</v>
+      </c>
       <c r="J25" s="12"/>
       <c r="K25" s="12" t="s">
         <v>174</v>
@@ -1863,7 +2054,7 @@
         <v>10</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="5" t="s">
         <v>11</v>
       </c>
@@ -1878,7 +2069,9 @@
       <c r="F26" s="12"/>
       <c r="G26" s="12"/>
       <c r="H26" s="12"/>
-      <c r="I26" s="12"/>
+      <c r="I26" s="12" t="s">
+        <v>213</v>
+      </c>
       <c r="J26" s="12"/>
       <c r="K26" s="12" t="s">
         <v>67</v>
@@ -1887,7 +2080,7 @@
         <v>12</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="5" t="s">
         <v>13</v>
       </c>
@@ -1902,7 +2095,9 @@
       <c r="F27" s="12"/>
       <c r="G27" s="12"/>
       <c r="H27" s="12"/>
-      <c r="I27" s="12"/>
+      <c r="I27" s="12" t="s">
+        <v>59</v>
+      </c>
       <c r="J27" s="12"/>
       <c r="K27" s="12" t="s">
         <v>172</v>
@@ -1911,7 +2106,7 @@
         <v>14</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="5" t="s">
         <v>15</v>
       </c>
@@ -1928,7 +2123,9 @@
       </c>
       <c r="G28" s="12"/>
       <c r="H28" s="12"/>
-      <c r="I28" s="12"/>
+      <c r="I28" s="12" t="s">
+        <v>74</v>
+      </c>
       <c r="J28" s="12"/>
       <c r="K28" s="12" t="s">
         <v>60</v>
@@ -1937,7 +2134,7 @@
         <v>16</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="5" t="s">
         <v>17</v>
       </c>
@@ -1952,16 +2149,18 @@
       <c r="F29" s="12"/>
       <c r="G29" s="12"/>
       <c r="H29" s="12"/>
-      <c r="I29" s="12"/>
+      <c r="I29" s="12" t="s">
+        <v>214</v>
+      </c>
       <c r="J29" s="12"/>
       <c r="K29" s="12" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="L29" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="5" t="s">
         <v>26</v>
       </c>
@@ -1976,7 +2175,9 @@
       <c r="F30" s="12"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
-      <c r="I30" s="12"/>
+      <c r="I30" s="12" t="s">
+        <v>62</v>
+      </c>
       <c r="J30" s="12"/>
       <c r="K30" s="12" t="s">
         <v>173</v>
@@ -1985,7 +2186,7 @@
         <v>27</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="5" t="s">
         <v>25</v>
       </c>
@@ -2000,14 +2201,16 @@
       <c r="F31" s="12"/>
       <c r="G31" s="12"/>
       <c r="H31" s="12"/>
-      <c r="I31" s="12"/>
+      <c r="I31" s="12" t="s">
+        <v>215</v>
+      </c>
       <c r="J31" s="12"/>
       <c r="K31" s="12" t="s">
         <v>174</v>
       </c>
       <c r="L31" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="5" t="s">
         <v>19</v>
       </c>
@@ -2022,7 +2225,9 @@
       <c r="F32" s="12"/>
       <c r="G32" s="12"/>
       <c r="H32" s="12"/>
-      <c r="I32" s="12"/>
+      <c r="I32" s="12" t="s">
+        <v>216</v>
+      </c>
       <c r="J32" s="12"/>
       <c r="K32" s="12" t="s">
         <v>175</v>
@@ -2031,7 +2236,7 @@
         <v>20</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="5" t="s">
         <v>21</v>
       </c>
@@ -2046,7 +2251,9 @@
       <c r="F33" s="12"/>
       <c r="G33" s="12"/>
       <c r="H33" s="12"/>
-      <c r="I33" s="12"/>
+      <c r="I33" s="12" t="s">
+        <v>237</v>
+      </c>
       <c r="J33" s="12"/>
       <c r="K33" s="12" t="s">
         <v>172</v>
@@ -2055,7 +2262,7 @@
         <v>22</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="5" t="s">
         <v>23</v>
       </c>
@@ -2070,14 +2277,16 @@
       <c r="F34" s="12"/>
       <c r="G34" s="12"/>
       <c r="H34" s="12"/>
-      <c r="I34" s="12"/>
+      <c r="I34" s="12" t="s">
+        <v>238</v>
+      </c>
       <c r="J34" s="12"/>
       <c r="K34" s="12" t="s">
         <v>67</v>
       </c>
       <c r="L34" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="5" t="s">
         <v>85</v>
       </c>
@@ -2092,7 +2301,9 @@
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
       <c r="H35" s="12"/>
-      <c r="I35" s="12"/>
+      <c r="I35" s="12" t="s">
+        <v>217</v>
+      </c>
       <c r="J35" s="12"/>
       <c r="K35" s="12" t="s">
         <v>176</v>
@@ -2101,7 +2312,7 @@
         <v>86</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="5" t="s">
         <v>28</v>
       </c>
@@ -2116,7 +2327,9 @@
       <c r="F36" s="12"/>
       <c r="G36" s="12"/>
       <c r="H36" s="12"/>
-      <c r="I36" s="12"/>
+      <c r="I36" s="12" t="s">
+        <v>250</v>
+      </c>
       <c r="J36" s="12"/>
       <c r="K36" s="12" t="s">
         <v>29</v>
@@ -2125,7 +2338,7 @@
         <v>30</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="5" t="s">
         <v>52</v>
       </c>
@@ -2140,14 +2353,16 @@
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
       <c r="H37" s="12"/>
-      <c r="I37" s="12"/>
+      <c r="I37" s="12" t="s">
+        <v>89</v>
+      </c>
       <c r="J37" s="12"/>
       <c r="K37" s="12" t="s">
         <v>67</v>
       </c>
       <c r="L37" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="4" t="s">
         <v>48</v>
       </c>
@@ -2163,7 +2378,7 @@
       <c r="K38" s="15"/>
       <c r="L38" s="10"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="5" t="s">
         <v>49</v>
       </c>
@@ -2178,14 +2393,16 @@
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
       <c r="H39" s="12"/>
-      <c r="I39" s="12"/>
+      <c r="I39" s="12" t="s">
+        <v>218</v>
+      </c>
       <c r="J39" s="12"/>
       <c r="K39" s="12" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="L39" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="40" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="40" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="5" t="s">
         <v>53</v>
       </c>
@@ -2200,14 +2417,16 @@
       <c r="F40" s="13"/>
       <c r="G40" s="13"/>
       <c r="H40" s="13"/>
-      <c r="I40" s="13"/>
+      <c r="I40" s="13" t="s">
+        <v>219</v>
+      </c>
       <c r="J40" s="12"/>
       <c r="K40" s="12" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="L40" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="41" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="41" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" s="5" t="s">
         <v>50</v>
       </c>
@@ -2222,14 +2441,16 @@
       <c r="F41" s="13"/>
       <c r="G41" s="13"/>
       <c r="H41" s="13"/>
-      <c r="I41" s="13"/>
+      <c r="I41" s="13" t="s">
+        <v>239</v>
+      </c>
       <c r="J41" s="12"/>
       <c r="K41" s="12" t="s">
         <v>177</v>
       </c>
       <c r="L41" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="42" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="42" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="5" t="s">
         <v>51</v>
       </c>
@@ -2244,14 +2465,16 @@
       <c r="F42" s="13"/>
       <c r="G42" s="13"/>
       <c r="H42" s="13"/>
-      <c r="I42" s="13"/>
+      <c r="I42" s="13" t="s">
+        <v>266</v>
+      </c>
       <c r="J42" s="12"/>
       <c r="K42" s="12" t="s">
         <v>178</v>
       </c>
       <c r="L42" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="5" t="s">
         <v>55</v>
       </c>
@@ -2266,14 +2489,16 @@
       <c r="F43" s="13"/>
       <c r="G43" s="13"/>
       <c r="H43" s="13"/>
-      <c r="I43" s="13"/>
+      <c r="I43" s="13" t="s">
+        <v>241</v>
+      </c>
       <c r="J43" s="12"/>
       <c r="K43" s="12" t="s">
         <v>179</v>
       </c>
       <c r="L43" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="44" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="44" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="5" t="s">
         <v>54</v>
       </c>
@@ -2288,14 +2513,16 @@
       <c r="F44" s="13"/>
       <c r="G44" s="13"/>
       <c r="H44" s="13"/>
-      <c r="I44" s="13"/>
+      <c r="I44" s="13" t="s">
+        <v>267</v>
+      </c>
       <c r="J44" s="12"/>
       <c r="K44" s="12" t="s">
         <v>180</v>
       </c>
       <c r="L44" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="45" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="45" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="5" t="s">
         <v>56</v>
       </c>
@@ -2310,14 +2537,16 @@
       <c r="F45" s="13"/>
       <c r="G45" s="13"/>
       <c r="H45" s="13"/>
-      <c r="I45" s="13"/>
+      <c r="I45" s="13" t="s">
+        <v>268</v>
+      </c>
       <c r="J45" s="12"/>
       <c r="K45" s="12" t="s">
         <v>181</v>
       </c>
       <c r="L45" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="46" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="46" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="4" t="s">
         <v>91</v>
       </c>
@@ -2333,7 +2562,7 @@
       <c r="K46" s="15"/>
       <c r="L46" s="10"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="47" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="47" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="5" t="s">
         <v>92</v>
       </c>
@@ -2348,16 +2577,18 @@
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
       <c r="H47" s="12"/>
-      <c r="I47" s="12"/>
+      <c r="I47" s="12" t="s">
+        <v>269</v>
+      </c>
       <c r="J47" s="12"/>
       <c r="K47" s="12" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="L47" s="9" t="s">
         <v>94</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="48" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="48" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="5" t="s">
         <v>93</v>
       </c>
@@ -2372,14 +2603,16 @@
       <c r="F48" s="13"/>
       <c r="G48" s="13"/>
       <c r="H48" s="13"/>
-      <c r="I48" s="13"/>
+      <c r="I48" s="13" t="s">
+        <v>270</v>
+      </c>
       <c r="J48" s="12"/>
       <c r="K48" s="12" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="L48" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="49" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="49" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="5" t="s">
         <v>95</v>
       </c>
@@ -2394,14 +2627,16 @@
       <c r="F49" s="13"/>
       <c r="G49" s="13"/>
       <c r="H49" s="13"/>
-      <c r="I49" s="13"/>
+      <c r="I49" s="13" t="s">
+        <v>271</v>
+      </c>
       <c r="J49" s="12"/>
       <c r="K49" s="12" t="s">
-        <v>221</v>
+        <v>208</v>
       </c>
       <c r="L49" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="50" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="50" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="5" t="s">
         <v>96</v>
       </c>
@@ -2416,14 +2651,16 @@
       <c r="F50" s="13"/>
       <c r="G50" s="13"/>
       <c r="H50" s="13"/>
-      <c r="I50" s="13"/>
+      <c r="I50" s="13" t="s">
+        <v>272</v>
+      </c>
       <c r="J50" s="12"/>
       <c r="K50" s="12" t="s">
-        <v>222</v>
+        <v>209</v>
       </c>
       <c r="L50" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="51" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="51" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="5" t="s">
         <v>97</v>
       </c>
@@ -2438,14 +2675,16 @@
       <c r="F51" s="13"/>
       <c r="G51" s="13"/>
       <c r="H51" s="13"/>
-      <c r="I51" s="13"/>
+      <c r="I51" s="13" t="s">
+        <v>220</v>
+      </c>
       <c r="J51" s="12"/>
       <c r="K51" s="12" t="s">
         <v>182</v>
       </c>
       <c r="L51" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="52" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="52" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="5" t="s">
         <v>98</v>
       </c>
@@ -2460,14 +2699,16 @@
       <c r="F52" s="13"/>
       <c r="G52" s="13"/>
       <c r="H52" s="13"/>
-      <c r="I52" s="13"/>
+      <c r="I52" s="13" t="s">
+        <v>221</v>
+      </c>
       <c r="J52" s="12"/>
       <c r="K52" s="12" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="L52" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="53" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="53" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="5" t="s">
         <v>106</v>
       </c>
@@ -2482,14 +2723,16 @@
       <c r="F53" s="13"/>
       <c r="G53" s="13"/>
       <c r="H53" s="13"/>
-      <c r="I53" s="13"/>
+      <c r="I53" s="13" t="s">
+        <v>273</v>
+      </c>
       <c r="J53" s="12"/>
       <c r="K53" s="12" t="s">
-        <v>223</v>
+        <v>210</v>
       </c>
       <c r="L53" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="54" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="54" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="5" t="s">
         <v>108</v>
       </c>
@@ -2504,10 +2747,12 @@
       <c r="F54" s="13"/>
       <c r="G54" s="13"/>
       <c r="H54" s="13"/>
-      <c r="I54" s="13"/>
+      <c r="I54" s="13" t="s">
+        <v>274</v>
+      </c>
       <c r="J54" s="12"/>
       <c r="K54" s="12" t="s">
-        <v>212</v>
+        <v>199</v>
       </c>
       <c r="L54" s="9"/>
     </row>
@@ -2518,6 +2763,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100841FCFF63B2DEE4FAB3ABDCB2B58E191" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6537ae6c172b48d8001feb3057ef3193">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f38bd768-81b4-450c-b73d-1a8fa3ba2722" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e79d1da23033c2d9c1658a7b9c3763cb" ns2:_="">
     <xsd:import namespace="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
@@ -2689,26 +2953,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5DB6742-085C-4A8F-8C68-EE166C6FD496}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0D3B35F-2651-4930-8D88-666C35501CF8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2724,22 +2987,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5DB6742-085C-4A8F-8C68-EE166C6FD496}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Corrections to landing, folding, general improvements
</commit_message>
<xml_diff>
--- a/Sizing/concepts_tabulations.xlsx
+++ b/Sizing/concepts_tabulations.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1321B93-04D9-4CA1-8592-7C23F99AA06B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CD77B38-E470-497C-AAFA-A79A758C3ABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Concepts" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" fullCalcOnLoad="true" iterate="true"/>
+  <calcPr calcId="191029" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="943" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="211">
   <si>
     <t>Deliverable</t>
   </si>
@@ -167,15 +167,6 @@
     <t>700nm Strike Mission Fuel Remaining [lb]</t>
   </si>
   <si>
-    <t>Combat Mission Max Range [nm]</t>
-  </si>
-  <si>
-    <t>Strike Mission Max Range [nm]</t>
-  </si>
-  <si>
-    <t>Ferry Mission Max Range [nm]</t>
-  </si>
-  <si>
     <t>Max Wing Loading [N/m2]</t>
   </si>
   <si>
@@ -221,500 +212,470 @@
     <t>5000</t>
   </si>
   <si>
+    <t>2000</t>
+  </si>
+  <si>
+    <t>29.3</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3.5672</t>
+  </si>
+  <si>
+    <t>0.33254</t>
+  </si>
+  <si>
+    <t>-0.027841</t>
+  </si>
+  <si>
+    <t>15.24</t>
+  </si>
+  <si>
+    <t>15000</t>
+  </si>
+  <si>
+    <t>Concept 2</t>
+  </si>
+  <si>
+    <t>Min Thrust Loading</t>
+  </si>
+  <si>
+    <t>Maximum Range [nm]</t>
+  </si>
+  <si>
+    <t>Maximum Endurance [min]</t>
+  </si>
+  <si>
+    <t>74.2354</t>
+  </si>
+  <si>
+    <t>184.2067</t>
+  </si>
+  <si>
+    <t>Unit Cost [millions]</t>
+  </si>
+  <si>
+    <t>For 500 aircraft</t>
+  </si>
+  <si>
+    <t>Spot Factor</t>
+  </si>
+  <si>
+    <t>Just from wing are projection</t>
+  </si>
+  <si>
+    <t>Fold Ratio</t>
+  </si>
+  <si>
+    <t>How much of the wing folds? 0.3193 for Hornet</t>
+  </si>
+  <si>
+    <t>Landing Speed [kt]</t>
+  </si>
+  <si>
+    <t>0.3193</t>
+  </si>
+  <si>
+    <t>Constraints</t>
+  </si>
+  <si>
+    <t>Mission Constraints</t>
+  </si>
+  <si>
+    <t>145kt Landing</t>
+  </si>
+  <si>
+    <t>We want all constraints to be less than 0 to be satisfied and a valid design</t>
+  </si>
+  <si>
+    <t>M1.6 Dash</t>
+  </si>
+  <si>
+    <t>M0.85 Dash</t>
+  </si>
+  <si>
+    <t>60ft Max Span</t>
+  </si>
+  <si>
+    <t>45 ton MTOW</t>
+  </si>
+  <si>
+    <t>8 Deg/s Sustained Turn</t>
+  </si>
+  <si>
+    <t>Max Sustained Turn Rate [deg/s]</t>
+  </si>
+  <si>
+    <t>Landing SEROC</t>
+  </si>
+  <si>
+    <t>Landing SEROC [ft/min]</t>
+  </si>
+  <si>
+    <t>Uses 1.3x stall (this is at MTOW)</t>
+  </si>
+  <si>
+    <t>F-16</t>
+  </si>
+  <si>
+    <t>732.2682</t>
+  </si>
+  <si>
+    <t>505.8509</t>
+  </si>
+  <si>
+    <t>911.0097</t>
+  </si>
+  <si>
+    <t>Temp</t>
+  </si>
+  <si>
+    <t>FA-18E</t>
+  </si>
+  <si>
+    <t>FA-18E Sized</t>
+  </si>
+  <si>
+    <t>1.2345</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>2500</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>0.5</t>
+  </si>
+  <si>
+    <t>4.5</t>
+  </si>
+  <si>
+    <t>0.33333</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>29.0546</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>-0.015748</t>
+  </si>
+  <si>
+    <t>88.2746</t>
+  </si>
+  <si>
+    <t>149.3268</t>
+  </si>
+  <si>
+    <t>1122.685</t>
+  </si>
+  <si>
+    <t>24.7998</t>
+  </si>
+  <si>
+    <t>2099.7648</t>
+  </si>
+  <si>
+    <t>351.725</t>
+  </si>
+  <si>
+    <t>1054.1178</t>
+  </si>
+  <si>
+    <t>791.8646</t>
+  </si>
+  <si>
+    <t>1221.1825</t>
+  </si>
+  <si>
+    <t>4817.0198</t>
+  </si>
+  <si>
+    <t>8.0252</t>
+  </si>
+  <si>
+    <t>36000</t>
+  </si>
+  <si>
+    <t>77969.4578</t>
+  </si>
+  <si>
+    <t>34331.4578</t>
+  </si>
+  <si>
+    <t>0.02984</t>
+  </si>
+  <si>
+    <t>-0.13367</t>
+  </si>
+  <si>
+    <t>-1.2454</t>
+  </si>
+  <si>
+    <t>1.6892</t>
+  </si>
+  <si>
+    <t>53.3798</t>
+  </si>
+  <si>
+    <t>93.1606</t>
+  </si>
+  <si>
+    <t>16.7378</t>
+  </si>
+  <si>
+    <t>7838.9933</t>
+  </si>
+  <si>
+    <t>1260.8647</t>
+  </si>
+  <si>
+    <t>0.53112</t>
+  </si>
+  <si>
+    <t>-0.035024</t>
+  </si>
+  <si>
+    <t>-0.059402</t>
+  </si>
+  <si>
+    <t>-0.13837</t>
+  </si>
+  <si>
+    <t>-0.06663</t>
+  </si>
+  <si>
+    <t>Combat Mission Max Radius [nm]</t>
+  </si>
+  <si>
+    <t>Strike Mission Max Radius [nm]</t>
+  </si>
+  <si>
+    <t>Ferry Mission Max Radius [nm]</t>
+  </si>
+  <si>
+    <t>77.4685</t>
+  </si>
+  <si>
+    <t>2.1483</t>
+  </si>
+  <si>
+    <t>1.6475</t>
+  </si>
+  <si>
+    <t>101.4981</t>
+  </si>
+  <si>
+    <t>59.7353</t>
+  </si>
+  <si>
+    <t>120.6075</t>
+  </si>
+  <si>
+    <t>705.2619</t>
+  </si>
+  <si>
+    <t>35.7197</t>
+  </si>
+  <si>
+    <t>22.7617</t>
+  </si>
+  <si>
+    <t>2269.1317</t>
+  </si>
+  <si>
+    <t>408.4451</t>
+  </si>
+  <si>
+    <t>6895.7839</t>
+  </si>
+  <si>
+    <t>920.9508</t>
+  </si>
+  <si>
+    <t>3262.6764</t>
+  </si>
+  <si>
+    <t>0.64563</t>
+  </si>
+  <si>
+    <t>9.4705</t>
+  </si>
+  <si>
+    <t>30376.2159</t>
+  </si>
+  <si>
+    <t>17.6619</t>
+  </si>
+  <si>
+    <t>7.4312</t>
+  </si>
+  <si>
+    <t>2.4712</t>
+  </si>
+  <si>
+    <t>64140.5612</t>
+  </si>
+  <si>
+    <t>26626.3453</t>
+  </si>
+  <si>
+    <t>4.9512</t>
+  </si>
+  <si>
+    <t>87.4471</t>
+  </si>
+  <si>
+    <t>-0.030318</t>
+  </si>
+  <si>
+    <t>-0.30001</t>
+  </si>
+  <si>
+    <t>-0.030361</t>
+  </si>
+  <si>
+    <t>-0.17008</t>
+  </si>
+  <si>
+    <t>-0.034238</t>
+  </si>
+  <si>
+    <t>-0.28733</t>
+  </si>
+  <si>
+    <t>-0.49064</t>
+  </si>
+  <si>
+    <t>-0.41052</t>
+  </si>
+  <si>
+    <t>73.6832</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>1.6589</t>
+  </si>
+  <si>
+    <t>139.947</t>
+  </si>
+  <si>
+    <t>53.7409</t>
+  </si>
+  <si>
+    <t>130.6523</t>
+  </si>
+  <si>
+    <t>1012.4536</t>
+  </si>
+  <si>
+    <t>27.0368</t>
+  </si>
+  <si>
+    <t>16.444</t>
+  </si>
+  <si>
+    <t>1691.3094</t>
+  </si>
+  <si>
+    <t>272.8649</t>
+  </si>
+  <si>
+    <t>607.4833</t>
+  </si>
+  <si>
+    <t>-4337.0929</t>
+  </si>
+  <si>
+    <t>6500.8437</t>
+  </si>
+  <si>
+    <t>0.69613</t>
+  </si>
+  <si>
+    <t>6.6602</t>
+  </si>
+  <si>
     <t>28450</t>
   </si>
   <si>
-    <t>2000</t>
-  </si>
-  <si>
     <t>12.05</t>
   </si>
   <si>
-    <t>29.3</t>
-  </si>
-  <si>
     <t>5.07</t>
   </si>
   <si>
     <t>1.686</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>3.5672</t>
-  </si>
-  <si>
-    <t>0.33254</t>
+    <t>59488.0861</t>
+  </si>
+  <si>
+    <t>23900.0861</t>
   </si>
   <si>
     <t>3.378</t>
   </si>
   <si>
-    <t>-0.027841</t>
-  </si>
-  <si>
     <t>40.7049</t>
   </si>
   <si>
-    <t>15.24</t>
-  </si>
-  <si>
-    <t>15000</t>
-  </si>
-  <si>
-    <t>Concept 2</t>
-  </si>
-  <si>
-    <t>Min Thrust Loading</t>
-  </si>
-  <si>
-    <t>Maximum Range [nm]</t>
-  </si>
-  <si>
-    <t>Maximum Endurance [min]</t>
-  </si>
-  <si>
-    <t>74.2354</t>
-  </si>
-  <si>
-    <t>184.2067</t>
-  </si>
-  <si>
-    <t>Unit Cost [millions]</t>
-  </si>
-  <si>
-    <t>For 500 aircraft</t>
-  </si>
-  <si>
-    <t>Spot Factor</t>
-  </si>
-  <si>
-    <t>Just from wing are projection</t>
-  </si>
-  <si>
-    <t>Fold Ratio</t>
-  </si>
-  <si>
-    <t>How much of the wing folds? 0.3193 for Hornet</t>
-  </si>
-  <si>
-    <t>Landing Speed [kt]</t>
-  </si>
-  <si>
-    <t>73.6832</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>0.3193</t>
-  </si>
-  <si>
-    <t>Constraints</t>
-  </si>
-  <si>
-    <t>Mission Constraints</t>
-  </si>
-  <si>
-    <t>145kt Landing</t>
-  </si>
-  <si>
-    <t>We want all constraints to be less than 0 to be satisfied and a valid design</t>
-  </si>
-  <si>
-    <t>M1.6 Dash</t>
-  </si>
-  <si>
-    <t>M0.85 Dash</t>
-  </si>
-  <si>
-    <t>60ft Max Span</t>
-  </si>
-  <si>
-    <t>45 ton MTOW</t>
+    <t>0.15245</t>
+  </si>
+  <si>
+    <t>-0.034848</t>
+  </si>
+  <si>
+    <t>-0.034213</t>
+  </si>
+  <si>
+    <t>-0.18249</t>
   </si>
   <si>
     <t>-0.3411</t>
   </si>
   <si>
-    <t>6500.8437</t>
-  </si>
-  <si>
-    <t>0.69613</t>
-  </si>
-  <si>
-    <t>59488.0861</t>
-  </si>
-  <si>
     <t>-0.33902</t>
   </si>
   <si>
-    <t>23900.0861</t>
-  </si>
-  <si>
-    <t>6.6602</t>
-  </si>
-  <si>
-    <t>8 Deg/s Sustained Turn</t>
-  </si>
-  <si>
-    <t>Max Sustained Turn Rate [deg/s]</t>
-  </si>
-  <si>
-    <t>Landing SEROC</t>
-  </si>
-  <si>
-    <t>Landing SEROC [ft/min]</t>
-  </si>
-  <si>
-    <t>1.6589</t>
-  </si>
-  <si>
-    <t>53.7409</t>
-  </si>
-  <si>
-    <t>130.6523</t>
-  </si>
-  <si>
-    <t>1691.3094</t>
-  </si>
-  <si>
-    <t>272.8649</t>
-  </si>
-  <si>
-    <t>607.4833</t>
-  </si>
-  <si>
-    <t>-4337.0929</t>
-  </si>
-  <si>
-    <t>0.15245</t>
-  </si>
-  <si>
-    <t>-0.18249</t>
-  </si>
-  <si>
     <t>-0.1089</t>
   </si>
   <si>
-    <t>Uses 1.3x stall (this is at MTOW)</t>
-  </si>
-  <si>
-    <t>F-16</t>
-  </si>
-  <si>
-    <t>732.2682</t>
-  </si>
-  <si>
-    <t>505.8509</t>
-  </si>
-  <si>
-    <t>911.0097</t>
-  </si>
-  <si>
-    <t>Temp</t>
-  </si>
-  <si>
-    <t>71.9985</t>
-  </si>
-  <si>
-    <t>2.2969</t>
-  </si>
-  <si>
-    <t>1.6675</t>
-  </si>
-  <si>
-    <t>63.0246</t>
-  </si>
-  <si>
-    <t>138.2653</t>
-  </si>
-  <si>
-    <t>0.72081</t>
-  </si>
-  <si>
-    <t>27600.4439</t>
-  </si>
-  <si>
-    <t>18.2623</t>
-  </si>
-  <si>
-    <t>7.6838</t>
-  </si>
-  <si>
-    <t>2.5552</t>
-  </si>
-  <si>
-    <t>57450.8461</t>
-  </si>
-  <si>
-    <t>22712.4022</t>
-  </si>
-  <si>
-    <t>5.1195</t>
-  </si>
-  <si>
-    <t>93.4938</t>
-  </si>
-  <si>
-    <t>-0.18621</t>
-  </si>
-  <si>
-    <t>-0.36166</t>
-  </si>
-  <si>
-    <t>-0.7396</t>
-  </si>
-  <si>
-    <t>170.5489</t>
-  </si>
-  <si>
-    <t>2480.9254</t>
-  </si>
-  <si>
-    <t>24.4519</t>
-  </si>
-  <si>
-    <t>16.167</t>
-  </si>
-  <si>
-    <t>0.1762</t>
-  </si>
-  <si>
-    <t>-0.034213</t>
-  </si>
-  <si>
-    <t>-3.9619</t>
-  </si>
-  <si>
-    <t>111.2554</t>
-  </si>
-  <si>
-    <t>1991.6565</t>
-  </si>
-  <si>
-    <t>36.0863</t>
-  </si>
-  <si>
-    <t>25.9986</t>
-  </si>
-  <si>
-    <t>2288.6897</t>
-  </si>
-  <si>
-    <t>426.0548</t>
-  </si>
-  <si>
-    <t>1116.1852</t>
-  </si>
-  <si>
-    <t>763.9237</t>
-  </si>
-  <si>
-    <t>1310.6232</t>
-  </si>
-  <si>
-    <t>5617.6582</t>
-  </si>
-  <si>
-    <t>5.7256</t>
-  </si>
-  <si>
-    <t>2733.3788</t>
-  </si>
-  <si>
-    <t>10.1343</t>
-  </si>
-  <si>
-    <t>-0.027845</t>
-  </si>
-  <si>
-    <t>-0.00020745</t>
-  </si>
-  <si>
-    <t>-0.23272</t>
-  </si>
-  <si>
-    <t>-0.045178</t>
-  </si>
-  <si>
-    <t>-0.0014053</t>
-  </si>
-  <si>
-    <t>-2.9833</t>
-  </si>
-  <si>
-    <t>FA-18E</t>
-  </si>
-  <si>
-    <t>FA-18E Sized</t>
-  </si>
-  <si>
-    <t>1.2345</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>2500</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>0.5</t>
-  </si>
-  <si>
-    <t>4.5</t>
-  </si>
-  <si>
-    <t>0.33333</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>29.0546</t>
-  </si>
-  <si>
-    <t>72</t>
-  </si>
-  <si>
-    <t>-0.015748</t>
-  </si>
-  <si>
-    <t>88.2746</t>
-  </si>
-  <si>
-    <t>111.3531</t>
-  </si>
-  <si>
-    <t>276.31</t>
-  </si>
-  <si>
-    <t>1.8286</t>
-  </si>
-  <si>
-    <t>149.3268</t>
-  </si>
-  <si>
-    <t>61.5607</t>
-  </si>
-  <si>
-    <t>168.1095</t>
-  </si>
-  <si>
-    <t>1122.685</t>
-  </si>
-  <si>
-    <t>24.7998</t>
-  </si>
-  <si>
-    <t>20.5136</t>
-  </si>
-  <si>
-    <t>2099.7648</t>
-  </si>
-  <si>
-    <t>351.725</t>
-  </si>
-  <si>
-    <t>1054.1178</t>
-  </si>
-  <si>
-    <t>791.8646</t>
-  </si>
-  <si>
-    <t>1221.1825</t>
-  </si>
-  <si>
-    <t>7414.0166</t>
-  </si>
-  <si>
-    <t>1243.0346</t>
-  </si>
-  <si>
-    <t>4817.0198</t>
-  </si>
-  <si>
-    <t>0.79668</t>
-  </si>
-  <si>
-    <t>8.0252</t>
-  </si>
-  <si>
-    <t>36000</t>
-  </si>
-  <si>
-    <t>77969.4578</t>
-  </si>
-  <si>
-    <t>34331.4578</t>
-  </si>
-  <si>
-    <t>-0.034529</t>
-  </si>
-  <si>
-    <t>0.02984</t>
-  </si>
-  <si>
-    <t>-0.16164</t>
-  </si>
-  <si>
-    <t>-0.25473</t>
-  </si>
-  <si>
-    <t>-0.13367</t>
-  </si>
-  <si>
-    <t>-0.4544</t>
-  </si>
-  <si>
-    <t>-1.2454</t>
-  </si>
-  <si>
-    <t>1.6892</t>
-  </si>
-  <si>
-    <t>53.3798</t>
-  </si>
-  <si>
-    <t>93.1606</t>
-  </si>
-  <si>
-    <t>16.7378</t>
-  </si>
-  <si>
-    <t>7838.9933</t>
-  </si>
-  <si>
-    <t>1260.8647</t>
-  </si>
-  <si>
-    <t>0.53112</t>
-  </si>
-  <si>
-    <t>-0.035024</t>
-  </si>
-  <si>
-    <t>-0.059402</t>
-  </si>
-  <si>
-    <t>-0.13837</t>
-  </si>
-  <si>
-    <t>-0.06663</t>
+    <t>-1.0249</t>
+  </si>
+  <si>
+    <t>Folded Span [ft]</t>
+  </si>
+  <si>
+    <t>35ft Fold Limit</t>
+  </si>
+  <si>
+    <t>12.6232</t>
+  </si>
+  <si>
+    <t>-0.63934</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -748,13 +709,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519242"/>
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407453"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -765,7 +726,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -879,59 +840,57 @@
       </bottom>
       <diagonal/>
     </border>
-    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -950,7 +909,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1101,7 +1060,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="true">
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1125,9 +1084,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="true">
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1151,7 +1110,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1186,7 +1145,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -1204,7 +1163,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="true">
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1229,7 +1188,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -1265,36 +1224,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
-  <dimension ref="A1:L54"/>
-  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
+  <dimension ref="A1:L56"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.796875" customWidth="true"/>
-    <col min="2" max="2" width="10.5" customWidth="true"/>
-    <col min="3" max="3" width="12.5" customWidth="true"/>
-    <col min="4" max="4" width="4.69921875" customWidth="true"/>
-    <col min="6" max="6" width="9.796875" customWidth="true"/>
-    <col min="11" max="11" width="10.5" customWidth="true"/>
-    <col min="12" max="12" width="106.796875" customWidth="true"/>
-    <col min="5" max="5" width="4.69921875" customWidth="true"/>
-    <col min="7" max="7" width="9.796875" customWidth="true"/>
-    <col min="8" max="8" width="9.796875" customWidth="true"/>
-    <col min="9" max="9" width="9.796875" customWidth="true"/>
-    <col min="10" max="10" width="9.796875" customWidth="true"/>
+    <col min="1" max="1" width="38.77734375" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="4" max="5" width="4.6640625" customWidth="1"/>
+    <col min="6" max="10" width="9.77734375" customWidth="1"/>
+    <col min="11" max="11" width="10.44140625" customWidth="1"/>
+    <col min="12" max="12" width="106.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" ht="15" thickBot="true" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>169</v>
+        <v>98</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>170</v>
+        <v>99</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>121</v>
+        <v>93</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>8</v>
@@ -1303,7 +1257,7 @@
         <v>1</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>2</v>
@@ -1315,13 +1269,13 @@
         <v>4</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>125</v>
+        <v>97</v>
       </c>
       <c r="L1" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1337,15 +1291,15 @@
       <c r="K2" s="3"/>
       <c r="L2" s="7"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>88</v>
+        <v>175</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="D3" s="11"/>
       <c r="E3" s="11"/>
@@ -1355,21 +1309,21 @@
       <c r="I3" s="12"/>
       <c r="J3" s="13"/>
       <c r="K3" s="13" t="s">
-        <v>183</v>
+        <v>112</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>89</v>
+        <v>176</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="11"/>
@@ -1379,21 +1333,21 @@
       <c r="I4" s="12"/>
       <c r="J4" s="13"/>
       <c r="K4" s="13" t="s">
-        <v>171</v>
+        <v>100</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="D5" s="11"/>
       <c r="E5" s="11"/>
@@ -1403,21 +1357,21 @@
       <c r="I5" s="12"/>
       <c r="J5" s="13"/>
       <c r="K5" s="13" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="L5" s="8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>34</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="D6" s="11"/>
       <c r="E6" s="11"/>
@@ -1427,21 +1381,21 @@
       <c r="I6" s="12"/>
       <c r="J6" s="13"/>
       <c r="K6" s="13" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="L6" s="8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>31</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>110</v>
+        <v>177</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="D7" s="11"/>
       <c r="E7" s="11"/>
@@ -1451,21 +1405,21 @@
       <c r="I7" s="12"/>
       <c r="J7" s="13"/>
       <c r="K7" s="13" t="s">
-        <v>213</v>
+        <v>129</v>
       </c>
       <c r="L7" s="8" t="s">
         <v>35</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>143</v>
+        <v>178</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="11"/>
@@ -1475,21 +1429,21 @@
       <c r="I8" s="12"/>
       <c r="J8" s="13"/>
       <c r="K8" s="13" t="s">
-        <v>187</v>
+        <v>113</v>
       </c>
       <c r="L8" s="8" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>36</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>111</v>
+        <v>179</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>129</v>
+        <v>147</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="11"/>
@@ -1499,19 +1453,19 @@
       <c r="I9" s="12"/>
       <c r="J9" s="13"/>
       <c r="K9" s="13" t="s">
-        <v>214</v>
+        <v>130</v>
       </c>
       <c r="L9" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>37</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>112</v>
+        <v>180</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>130</v>
+        <v>148</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="11"/>
@@ -1521,19 +1475,19 @@
       <c r="I10" s="12"/>
       <c r="J10" s="13"/>
       <c r="K10" s="13" t="s">
-        <v>215</v>
+        <v>131</v>
       </c>
       <c r="L10" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>144</v>
+        <v>181</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
@@ -1543,19 +1497,19 @@
       <c r="I11" s="12"/>
       <c r="J11" s="13"/>
       <c r="K11" s="13" t="s">
-        <v>190</v>
+        <v>114</v>
       </c>
       <c r="L11" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>38</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>145</v>
+        <v>182</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="11"/>
@@ -1565,19 +1519,19 @@
       <c r="I12" s="12"/>
       <c r="J12" s="13"/>
       <c r="K12" s="13" t="s">
-        <v>191</v>
+        <v>115</v>
       </c>
       <c r="L12" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>146</v>
+        <v>183</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="11"/>
@@ -1587,19 +1541,19 @@
       <c r="I13" s="12"/>
       <c r="J13" s="13"/>
       <c r="K13" s="13" t="s">
-        <v>216</v>
+        <v>132</v>
       </c>
       <c r="L13" s="8"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>113</v>
+        <v>184</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D14" s="11"/>
       <c r="E14" s="11"/>
@@ -1609,21 +1563,21 @@
       <c r="I14" s="12"/>
       <c r="J14" s="12"/>
       <c r="K14" s="12" t="s">
-        <v>193</v>
+        <v>116</v>
       </c>
       <c r="L14" s="9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>114</v>
+        <v>185</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="11"/>
@@ -1633,21 +1587,21 @@
       <c r="I15" s="12"/>
       <c r="J15" s="12"/>
       <c r="K15" s="12" t="s">
-        <v>194</v>
+        <v>117</v>
       </c>
       <c r="L15" s="9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>43</v>
+        <v>140</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>122</v>
+        <v>94</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>156</v>
+        <v>94</v>
       </c>
       <c r="D16" s="11"/>
       <c r="E16" s="11"/>
@@ -1657,19 +1611,19 @@
       <c r="I16" s="12"/>
       <c r="J16" s="12"/>
       <c r="K16" s="12" t="s">
-        <v>195</v>
+        <v>118</v>
       </c>
       <c r="L16" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>44</v>
+        <v>141</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>123</v>
+        <v>95</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>157</v>
+        <v>95</v>
       </c>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
@@ -1679,19 +1633,19 @@
       <c r="I17" s="12"/>
       <c r="J17" s="12"/>
       <c r="K17" s="12" t="s">
-        <v>196</v>
+        <v>119</v>
       </c>
       <c r="L17" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>45</v>
+        <v>142</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>124</v>
+        <v>96</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>158</v>
+        <v>96</v>
       </c>
       <c r="D18" s="11"/>
       <c r="E18" s="11"/>
@@ -1701,19 +1655,19 @@
       <c r="I18" s="12"/>
       <c r="J18" s="12"/>
       <c r="K18" s="12" t="s">
-        <v>197</v>
+        <v>120</v>
       </c>
       <c r="L18" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>41</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>115</v>
+        <v>186</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
@@ -1723,19 +1677,19 @@
       <c r="I19" s="12"/>
       <c r="J19" s="12"/>
       <c r="K19" s="12" t="s">
-        <v>217</v>
+        <v>133</v>
       </c>
       <c r="L19" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>42</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>116</v>
+        <v>187</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
@@ -1745,19 +1699,19 @@
       <c r="I20" s="12"/>
       <c r="J20" s="12"/>
       <c r="K20" s="12" t="s">
-        <v>218</v>
+        <v>134</v>
       </c>
       <c r="L20" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>100</v>
+        <v>188</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="D21" s="11"/>
       <c r="E21" s="11"/>
@@ -1767,21 +1721,21 @@
       <c r="I21" s="12"/>
       <c r="J21" s="12"/>
       <c r="K21" s="12" t="s">
-        <v>200</v>
+        <v>121</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>101</v>
+        <v>189</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>131</v>
+        <v>157</v>
       </c>
       <c r="D22" s="11"/>
       <c r="E22" s="11"/>
@@ -1791,21 +1745,21 @@
       <c r="I22" s="12"/>
       <c r="J22" s="12"/>
       <c r="K22" s="12" t="s">
-        <v>219</v>
+        <v>135</v>
       </c>
       <c r="L22" s="9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>6</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>105</v>
+        <v>190</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="D23" s="11"/>
       <c r="E23" s="11"/>
@@ -1815,13 +1769,13 @@
       <c r="I23" s="12"/>
       <c r="J23" s="12"/>
       <c r="K23" s="12" t="s">
-        <v>202</v>
+        <v>122</v>
       </c>
       <c r="L23" s="9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>24</v>
       </c>
@@ -1837,41 +1791,41 @@
       <c r="K24" s="15"/>
       <c r="L24" s="10"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D25" s="11"/>
       <c r="E25" s="11"/>
       <c r="F25" s="12" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="12"/>
       <c r="I25" s="12"/>
       <c r="J25" s="12"/>
       <c r="K25" s="12" t="s">
-        <v>174</v>
+        <v>103</v>
       </c>
       <c r="L25" s="9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D26" s="11"/>
       <c r="E26" s="11"/>
@@ -1881,21 +1835,21 @@
       <c r="I26" s="12"/>
       <c r="J26" s="12"/>
       <c r="K26" s="12" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="L26" s="9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>13</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D27" s="11"/>
       <c r="E27" s="11"/>
@@ -1905,47 +1859,47 @@
       <c r="I27" s="12"/>
       <c r="J27" s="12"/>
       <c r="K27" s="12" t="s">
-        <v>172</v>
+        <v>101</v>
       </c>
       <c r="L27" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>15</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D28" s="11"/>
       <c r="E28" s="11"/>
       <c r="F28" s="12" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="G28" s="12"/>
       <c r="H28" s="12"/>
       <c r="I28" s="12"/>
       <c r="J28" s="12"/>
       <c r="K28" s="12" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="L28" s="9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>17</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>61</v>
+        <v>191</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>132</v>
+        <v>159</v>
       </c>
       <c r="D29" s="11"/>
       <c r="E29" s="11"/>
@@ -1955,21 +1909,21 @@
       <c r="I29" s="12"/>
       <c r="J29" s="12"/>
       <c r="K29" s="12" t="s">
-        <v>203</v>
+        <v>123</v>
       </c>
       <c r="L29" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D30" s="11"/>
       <c r="E30" s="11"/>
@@ -1979,21 +1933,21 @@
       <c r="I30" s="12"/>
       <c r="J30" s="12"/>
       <c r="K30" s="12" t="s">
-        <v>173</v>
+        <v>102</v>
       </c>
       <c r="L30" s="9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>25</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>63</v>
+        <v>192</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>133</v>
+        <v>160</v>
       </c>
       <c r="D31" s="11"/>
       <c r="E31" s="11"/>
@@ -2003,19 +1957,19 @@
       <c r="I31" s="12"/>
       <c r="J31" s="12"/>
       <c r="K31" s="12" t="s">
-        <v>174</v>
+        <v>103</v>
       </c>
       <c r="L31" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>19</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D32" s="11"/>
       <c r="E32" s="11"/>
@@ -2025,21 +1979,21 @@
       <c r="I32" s="12"/>
       <c r="J32" s="12"/>
       <c r="K32" s="12" t="s">
-        <v>175</v>
+        <v>104</v>
       </c>
       <c r="L32" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>21</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>65</v>
+        <v>193</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>134</v>
+        <v>161</v>
       </c>
       <c r="D33" s="11"/>
       <c r="E33" s="11"/>
@@ -2049,21 +2003,21 @@
       <c r="I33" s="12"/>
       <c r="J33" s="12"/>
       <c r="K33" s="12" t="s">
-        <v>172</v>
+        <v>101</v>
       </c>
       <c r="L33" s="9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>66</v>
+        <v>194</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>135</v>
+        <v>162</v>
       </c>
       <c r="D34" s="11"/>
       <c r="E34" s="11"/>
@@ -2073,19 +2027,19 @@
       <c r="I34" s="12"/>
       <c r="J34" s="12"/>
       <c r="K34" s="12" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="L34" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="D35" s="11"/>
       <c r="E35" s="11"/>
@@ -2095,13 +2049,13 @@
       <c r="I35" s="12"/>
       <c r="J35" s="12"/>
       <c r="K35" s="12" t="s">
-        <v>176</v>
+        <v>105</v>
       </c>
       <c r="L35" s="9" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>28</v>
       </c>
@@ -2125,15 +2079,15 @@
         <v>30</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="D37" s="11"/>
       <c r="E37" s="11"/>
@@ -2143,13 +2097,13 @@
       <c r="I37" s="12"/>
       <c r="J37" s="12"/>
       <c r="K37" s="12" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="L37" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B38" s="15"/>
       <c r="C38" s="15"/>
@@ -2163,15 +2117,15 @@
       <c r="K38" s="15"/>
       <c r="L38" s="10"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>102</v>
+        <v>195</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>136</v>
+        <v>163</v>
       </c>
       <c r="D39" s="11"/>
       <c r="E39" s="11"/>
@@ -2181,19 +2135,19 @@
       <c r="I39" s="12"/>
       <c r="J39" s="12"/>
       <c r="K39" s="12" t="s">
-        <v>204</v>
+        <v>124</v>
       </c>
       <c r="L39" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="40" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>137</v>
+        <v>196</v>
+      </c>
+      <c r="C40" s="11" t="s">
+        <v>164</v>
       </c>
       <c r="D40" s="14"/>
       <c r="E40" s="14"/>
@@ -2203,19 +2157,19 @@
       <c r="I40" s="13"/>
       <c r="J40" s="12"/>
       <c r="K40" s="12" t="s">
-        <v>205</v>
+        <v>125</v>
       </c>
       <c r="L40" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="41" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="C41" s="14" t="s">
-        <v>68</v>
+        <v>61</v>
+      </c>
+      <c r="C41" s="11" t="s">
+        <v>61</v>
       </c>
       <c r="D41" s="14"/>
       <c r="E41" s="14"/>
@@ -2225,19 +2179,19 @@
       <c r="I41" s="13"/>
       <c r="J41" s="12"/>
       <c r="K41" s="12" t="s">
-        <v>177</v>
+        <v>106</v>
       </c>
       <c r="L41" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="42" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="C42" s="14" t="s">
-        <v>69</v>
+        <v>62</v>
+      </c>
+      <c r="C42" s="11" t="s">
+        <v>62</v>
       </c>
       <c r="D42" s="14"/>
       <c r="E42" s="14"/>
@@ -2247,19 +2201,19 @@
       <c r="I42" s="13"/>
       <c r="J42" s="12"/>
       <c r="K42" s="12" t="s">
-        <v>178</v>
+        <v>107</v>
       </c>
       <c r="L42" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C43" s="14" t="s">
-        <v>138</v>
+        <v>197</v>
+      </c>
+      <c r="C43" s="11" t="s">
+        <v>165</v>
       </c>
       <c r="D43" s="14"/>
       <c r="E43" s="14"/>
@@ -2269,20 +2223,18 @@
       <c r="I43" s="13"/>
       <c r="J43" s="12"/>
       <c r="K43" s="12" t="s">
-        <v>179</v>
+        <v>108</v>
       </c>
       <c r="L43" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="44" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
-        <v>54</v>
+        <v>207</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="C44" s="14" t="s">
-        <v>163</v>
-      </c>
+        <v>209</v>
+      </c>
+      <c r="C44" s="11"/>
       <c r="D44" s="14"/>
       <c r="E44" s="14"/>
       <c r="F44" s="13"/>
@@ -2290,20 +2242,18 @@
       <c r="H44" s="13"/>
       <c r="I44" s="13"/>
       <c r="J44" s="12"/>
-      <c r="K44" s="12" t="s">
-        <v>180</v>
-      </c>
+      <c r="K44" s="12"/>
       <c r="L44" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="45" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="C45" s="14" t="s">
-        <v>139</v>
+        <v>63</v>
+      </c>
+      <c r="C45" s="11" t="s">
+        <v>63</v>
       </c>
       <c r="D45" s="14"/>
       <c r="E45" s="14"/>
@@ -2313,81 +2263,81 @@
       <c r="I45" s="13"/>
       <c r="J45" s="12"/>
       <c r="K45" s="12" t="s">
-        <v>181</v>
+        <v>109</v>
       </c>
       <c r="L45" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="46" x14ac:dyDescent="0.3">
-      <c r="A46" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B46" s="15"/>
-      <c r="C46" s="15"/>
-      <c r="D46" s="15"/>
-      <c r="E46" s="15"/>
-      <c r="F46" s="15"/>
-      <c r="G46" s="15"/>
-      <c r="H46" s="15"/>
-      <c r="I46" s="15"/>
-      <c r="J46" s="15"/>
-      <c r="K46" s="15"/>
-      <c r="L46" s="10"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="47" x14ac:dyDescent="0.3">
-      <c r="A47" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="B47" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="C47" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="D47" s="11"/>
-      <c r="E47" s="11"/>
-      <c r="F47" s="12"/>
-      <c r="G47" s="12"/>
-      <c r="H47" s="12"/>
-      <c r="I47" s="12"/>
-      <c r="J47" s="12"/>
-      <c r="K47" s="12" t="s">
-        <v>220</v>
-      </c>
-      <c r="L47" s="9" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="48" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A46" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="C46" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="D46" s="14"/>
+      <c r="E46" s="14"/>
+      <c r="F46" s="13"/>
+      <c r="G46" s="13"/>
+      <c r="H46" s="13"/>
+      <c r="I46" s="13"/>
+      <c r="J46" s="12"/>
+      <c r="K46" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="L46" s="9"/>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A47" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B47" s="15"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="15"/>
+      <c r="H47" s="15"/>
+      <c r="I47" s="15"/>
+      <c r="J47" s="15"/>
+      <c r="K47" s="15"/>
+      <c r="L47" s="10"/>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="C48" s="14" t="s">
-        <v>165</v>
-      </c>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="13"/>
-      <c r="G48" s="13"/>
-      <c r="H48" s="13"/>
-      <c r="I48" s="13"/>
+        <v>199</v>
+      </c>
+      <c r="C48" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="D48" s="11"/>
+      <c r="E48" s="11"/>
+      <c r="F48" s="12"/>
+      <c r="G48" s="12"/>
+      <c r="H48" s="12"/>
+      <c r="I48" s="12"/>
       <c r="J48" s="12"/>
       <c r="K48" s="12" t="s">
-        <v>207</v>
-      </c>
-      <c r="L48" s="9"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="49" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+      <c r="L48" s="9" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>148</v>
-      </c>
-      <c r="C49" s="14" t="s">
-        <v>166</v>
+        <v>200</v>
+      </c>
+      <c r="C49" s="11" t="s">
+        <v>168</v>
       </c>
       <c r="D49" s="14"/>
       <c r="E49" s="14"/>
@@ -2397,19 +2347,19 @@
       <c r="I49" s="13"/>
       <c r="J49" s="12"/>
       <c r="K49" s="12" t="s">
-        <v>221</v>
+        <v>126</v>
       </c>
       <c r="L49" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="50" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="C50" s="14" t="s">
-        <v>140</v>
+        <v>201</v>
+      </c>
+      <c r="C50" s="11" t="s">
+        <v>169</v>
       </c>
       <c r="D50" s="14"/>
       <c r="E50" s="14"/>
@@ -2419,19 +2369,19 @@
       <c r="I50" s="13"/>
       <c r="J50" s="12"/>
       <c r="K50" s="12" t="s">
-        <v>222</v>
+        <v>137</v>
       </c>
       <c r="L50" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="51" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="C51" s="14" t="s">
-        <v>167</v>
+        <v>202</v>
+      </c>
+      <c r="C51" s="11" t="s">
+        <v>170</v>
       </c>
       <c r="D51" s="14"/>
       <c r="E51" s="14"/>
@@ -2441,19 +2391,19 @@
       <c r="I51" s="13"/>
       <c r="J51" s="12"/>
       <c r="K51" s="12" t="s">
-        <v>182</v>
+        <v>138</v>
       </c>
       <c r="L51" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="52" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="C52" s="14" t="s">
-        <v>141</v>
+        <v>203</v>
+      </c>
+      <c r="C52" s="11" t="s">
+        <v>171</v>
       </c>
       <c r="D52" s="14"/>
       <c r="E52" s="14"/>
@@ -2463,19 +2413,19 @@
       <c r="I52" s="13"/>
       <c r="J52" s="12"/>
       <c r="K52" s="12" t="s">
-        <v>210</v>
+        <v>111</v>
       </c>
       <c r="L52" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="53" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="C53" s="14" t="s">
-        <v>142</v>
+        <v>204</v>
+      </c>
+      <c r="C53" s="11" t="s">
+        <v>172</v>
       </c>
       <c r="D53" s="14"/>
       <c r="E53" s="14"/>
@@ -2485,19 +2435,19 @@
       <c r="I53" s="13"/>
       <c r="J53" s="12"/>
       <c r="K53" s="12" t="s">
-        <v>223</v>
+        <v>127</v>
       </c>
       <c r="L53" s="9"/>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="54" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="C54" s="14" t="s">
-        <v>168</v>
+        <v>205</v>
+      </c>
+      <c r="C54" s="11" t="s">
+        <v>173</v>
       </c>
       <c r="D54" s="14"/>
       <c r="E54" s="14"/>
@@ -2507,9 +2457,48 @@
       <c r="I54" s="13"/>
       <c r="J54" s="12"/>
       <c r="K54" s="12" t="s">
-        <v>212</v>
+        <v>139</v>
       </c>
       <c r="L54" s="9"/>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A55" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B55" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="C55" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="D55" s="14"/>
+      <c r="E55" s="14"/>
+      <c r="F55" s="13"/>
+      <c r="G55" s="13"/>
+      <c r="H55" s="13"/>
+      <c r="I55" s="13"/>
+      <c r="J55" s="12"/>
+      <c r="K55" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="L55" s="9"/>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A56" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="C56" s="11"/>
+      <c r="D56" s="14"/>
+      <c r="E56" s="14"/>
+      <c r="F56" s="13"/>
+      <c r="G56" s="13"/>
+      <c r="H56" s="13"/>
+      <c r="I56" s="13"/>
+      <c r="J56" s="12"/>
+      <c r="K56" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2518,6 +2507,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100841FCFF63B2DEE4FAB3ABDCB2B58E191" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6537ae6c172b48d8001feb3057ef3193">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f38bd768-81b4-450c-b73d-1a8fa3ba2722" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e79d1da23033c2d9c1658a7b9c3763cb" ns2:_="">
     <xsd:import namespace="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
@@ -2689,26 +2697,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5DB6742-085C-4A8F-8C68-EE166C6FD496}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0D3B35F-2651-4930-8D88-666C35501CF8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2724,22 +2731,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5DB6742-085C-4A8F-8C68-EE166C6FD496}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
more changes to excel
</commit_message>
<xml_diff>
--- a/Sizing/concepts_tabulations.xlsx
+++ b/Sizing/concepts_tabulations.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -10,12 +10,12 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CD77B38-E470-497C-AAFA-A79A758C3ABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
     <sheet name="Concepts" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="true" iterate="true"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="482" uniqueCount="246">
   <si>
     <t>Deliverable</t>
   </si>
@@ -669,13 +669,118 @@
   </si>
   <si>
     <t>-0.63934</t>
+  </si>
+  <si>
+    <t>77.3332</t>
+  </si>
+  <si>
+    <t>2.1639</t>
+  </si>
+  <si>
+    <t>1.648</t>
+  </si>
+  <si>
+    <t>101.0453</t>
+  </si>
+  <si>
+    <t>59.8707</t>
+  </si>
+  <si>
+    <t>121.0116</t>
+  </si>
+  <si>
+    <t>713.9192</t>
+  </si>
+  <si>
+    <t>35.8702</t>
+  </si>
+  <si>
+    <t>22.9032</t>
+  </si>
+  <si>
+    <t>2276.107</t>
+  </si>
+  <si>
+    <t>410.0479</t>
+  </si>
+  <si>
+    <t>6882.946</t>
+  </si>
+  <si>
+    <t>929.6226</t>
+  </si>
+  <si>
+    <t>3230.7634</t>
+  </si>
+  <si>
+    <t>0.64733</t>
+  </si>
+  <si>
+    <t>9.5119</t>
+  </si>
+  <si>
+    <t>30306.9449</t>
+  </si>
+  <si>
+    <t>17.7256</t>
+  </si>
+  <si>
+    <t>7.458</t>
+  </si>
+  <si>
+    <t>2.4801</t>
+  </si>
+  <si>
+    <t>63972.4653</t>
+  </si>
+  <si>
+    <t>26527.5204</t>
+  </si>
+  <si>
+    <t>4.9691</t>
+  </si>
+  <si>
+    <t>18.5688</t>
+  </si>
+  <si>
+    <t>-0.027912</t>
+  </si>
+  <si>
+    <t>88.0794</t>
+  </si>
+  <si>
+    <t>-0.030674</t>
+  </si>
+  <si>
+    <t>-0.30314</t>
+  </si>
+  <si>
+    <t>-0.030657</t>
+  </si>
+  <si>
+    <t>-0.1705</t>
+  </si>
+  <si>
+    <t>-0.030753</t>
+  </si>
+  <si>
+    <t>-0.28919</t>
+  </si>
+  <si>
+    <t>-0.50032</t>
+  </si>
+  <si>
+    <t>-0.42784</t>
+  </si>
+  <si>
+    <t>-0.46946</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -709,13 +814,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
+        <fgColor theme="4" tint="0.39997558519242"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="0" tint="-0.14999847407453"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -726,7 +831,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -840,57 +945,59 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -909,7 +1016,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1060,7 +1167,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1084,9 +1191,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1110,7 +1217,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1145,7 +1252,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -1163,7 +1270,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1188,7 +1295,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -1224,20 +1331,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
   <dimension ref="A1:L56"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.77734375" customWidth="1"/>
-    <col min="2" max="2" width="10.44140625" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" customWidth="1"/>
-    <col min="4" max="5" width="4.6640625" customWidth="1"/>
-    <col min="6" max="10" width="9.77734375" customWidth="1"/>
-    <col min="11" max="11" width="10.44140625" customWidth="1"/>
-    <col min="12" max="12" width="106.77734375" customWidth="1"/>
+    <col min="1" max="1" width="38.796875" customWidth="true"/>
+    <col min="2" max="2" width="10.5" customWidth="true"/>
+    <col min="3" max="3" width="12.5" customWidth="true"/>
+    <col min="4" max="4" width="4.69921875" customWidth="true"/>
+    <col min="6" max="6" width="9.796875" customWidth="true"/>
+    <col min="11" max="11" width="10.5" customWidth="true"/>
+    <col min="12" max="12" width="106.796875" customWidth="true"/>
+    <col min="5" max="5" width="4.69921875" customWidth="true"/>
+    <col min="7" max="7" width="9.796875" customWidth="true"/>
+    <col min="8" max="8" width="9.796875" customWidth="true"/>
+    <col min="9" max="9" width="9.796875" customWidth="true"/>
+    <col min="10" max="10" width="9.796875" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" ht="15" thickBot="true" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1275,7 +1387,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1291,7 +1403,7 @@
       <c r="K2" s="3"/>
       <c r="L2" s="7"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>72</v>
       </c>
@@ -1299,7 +1411,7 @@
         <v>175</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>143</v>
+        <v>211</v>
       </c>
       <c r="D3" s="11"/>
       <c r="E3" s="11"/>
@@ -1315,7 +1427,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>74</v>
       </c>
@@ -1323,7 +1435,7 @@
         <v>176</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>144</v>
+        <v>212</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="11"/>
@@ -1339,7 +1451,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
@@ -1363,7 +1475,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>34</v>
       </c>
@@ -1387,7 +1499,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>31</v>
       </c>
@@ -1395,7 +1507,7 @@
         <v>177</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>145</v>
+        <v>213</v>
       </c>
       <c r="D7" s="11"/>
       <c r="E7" s="11"/>
@@ -1411,7 +1523,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>78</v>
       </c>
@@ -1419,7 +1531,7 @@
         <v>178</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>146</v>
+        <v>214</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="11"/>
@@ -1435,7 +1547,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>36</v>
       </c>
@@ -1443,7 +1555,7 @@
         <v>179</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>147</v>
+        <v>215</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="11"/>
@@ -1457,7 +1569,7 @@
       </c>
       <c r="L9" s="8"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>37</v>
       </c>
@@ -1465,7 +1577,7 @@
         <v>180</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>148</v>
+        <v>216</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="11"/>
@@ -1479,7 +1591,7 @@
       </c>
       <c r="L10" s="8"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>91</v>
       </c>
@@ -1487,7 +1599,7 @@
         <v>181</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>149</v>
+        <v>217</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
@@ -1501,7 +1613,7 @@
       </c>
       <c r="L11" s="8"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>38</v>
       </c>
@@ -1509,7 +1621,7 @@
         <v>182</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>150</v>
+        <v>218</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="11"/>
@@ -1523,7 +1635,7 @@
       </c>
       <c r="L12" s="8"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>89</v>
       </c>
@@ -1531,7 +1643,7 @@
         <v>183</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>151</v>
+        <v>219</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="11"/>
@@ -1545,7 +1657,7 @@
       </c>
       <c r="L13" s="8"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>68</v>
       </c>
@@ -1553,7 +1665,7 @@
         <v>184</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>152</v>
+        <v>220</v>
       </c>
       <c r="D14" s="11"/>
       <c r="E14" s="11"/>
@@ -1569,7 +1681,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>69</v>
       </c>
@@ -1577,7 +1689,7 @@
         <v>185</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>153</v>
+        <v>221</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="11"/>
@@ -1593,7 +1705,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>140</v>
       </c>
@@ -1615,7 +1727,7 @@
       </c>
       <c r="L16" s="9"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>141</v>
       </c>
@@ -1637,7 +1749,7 @@
       </c>
       <c r="L17" s="9"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>142</v>
       </c>
@@ -1659,7 +1771,7 @@
       </c>
       <c r="L18" s="9"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>41</v>
       </c>
@@ -1667,7 +1779,7 @@
         <v>186</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>154</v>
+        <v>222</v>
       </c>
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
@@ -1681,7 +1793,7 @@
       </c>
       <c r="L19" s="9"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>42</v>
       </c>
@@ -1689,7 +1801,7 @@
         <v>187</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>155</v>
+        <v>223</v>
       </c>
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
@@ -1703,7 +1815,7 @@
       </c>
       <c r="L20" s="9"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>43</v>
       </c>
@@ -1711,7 +1823,7 @@
         <v>188</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>156</v>
+        <v>224</v>
       </c>
       <c r="D21" s="11"/>
       <c r="E21" s="11"/>
@@ -1727,7 +1839,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>67</v>
       </c>
@@ -1735,7 +1847,7 @@
         <v>189</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>157</v>
+        <v>225</v>
       </c>
       <c r="D22" s="11"/>
       <c r="E22" s="11"/>
@@ -1751,7 +1863,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>6</v>
       </c>
@@ -1759,7 +1871,7 @@
         <v>190</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>158</v>
+        <v>226</v>
       </c>
       <c r="D23" s="11"/>
       <c r="E23" s="11"/>
@@ -1775,7 +1887,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>24</v>
       </c>
@@ -1791,7 +1903,7 @@
       <c r="K24" s="15"/>
       <c r="L24" s="10"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>9</v>
       </c>
@@ -1817,7 +1929,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>11</v>
       </c>
@@ -1841,7 +1953,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>13</v>
       </c>
@@ -1865,7 +1977,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>15</v>
       </c>
@@ -1891,7 +2003,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>17</v>
       </c>
@@ -1899,7 +2011,7 @@
         <v>191</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>159</v>
+        <v>227</v>
       </c>
       <c r="D29" s="11"/>
       <c r="E29" s="11"/>
@@ -1915,7 +2027,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>26</v>
       </c>
@@ -1939,7 +2051,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>25</v>
       </c>
@@ -1947,7 +2059,7 @@
         <v>192</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>160</v>
+        <v>228</v>
       </c>
       <c r="D31" s="11"/>
       <c r="E31" s="11"/>
@@ -1961,7 +2073,7 @@
       </c>
       <c r="L31" s="9"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>19</v>
       </c>
@@ -1985,7 +2097,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>21</v>
       </c>
@@ -1993,7 +2105,7 @@
         <v>193</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>161</v>
+        <v>229</v>
       </c>
       <c r="D33" s="11"/>
       <c r="E33" s="11"/>
@@ -2009,7 +2121,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>23</v>
       </c>
@@ -2017,7 +2129,7 @@
         <v>194</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>162</v>
+        <v>230</v>
       </c>
       <c r="D34" s="11"/>
       <c r="E34" s="11"/>
@@ -2031,7 +2143,7 @@
       </c>
       <c r="L34" s="9"/>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>76</v>
       </c>
@@ -2055,7 +2167,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>28</v>
       </c>
@@ -2079,7 +2191,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>49</v>
       </c>
@@ -2101,7 +2213,7 @@
       </c>
       <c r="L37" s="9"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>45</v>
       </c>
@@ -2117,7 +2229,7 @@
       <c r="K38" s="15"/>
       <c r="L38" s="10"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>46</v>
       </c>
@@ -2125,7 +2237,7 @@
         <v>195</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>163</v>
+        <v>231</v>
       </c>
       <c r="D39" s="11"/>
       <c r="E39" s="11"/>
@@ -2139,7 +2251,7 @@
       </c>
       <c r="L39" s="9"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="40" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>50</v>
       </c>
@@ -2147,7 +2259,7 @@
         <v>196</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>164</v>
+        <v>232</v>
       </c>
       <c r="D40" s="14"/>
       <c r="E40" s="14"/>
@@ -2161,7 +2273,7 @@
       </c>
       <c r="L40" s="9"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="41" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>47</v>
       </c>
@@ -2183,7 +2295,7 @@
       </c>
       <c r="L41" s="9"/>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="42" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>48</v>
       </c>
@@ -2205,7 +2317,7 @@
       </c>
       <c r="L42" s="9"/>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>52</v>
       </c>
@@ -2213,7 +2325,7 @@
         <v>197</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>165</v>
+        <v>233</v>
       </c>
       <c r="D43" s="14"/>
       <c r="E43" s="14"/>
@@ -2227,14 +2339,16 @@
       </c>
       <c r="L43" s="9"/>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="44" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>207</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="C44" s="11"/>
+      <c r="C44" s="11" t="s">
+        <v>234</v>
+      </c>
       <c r="D44" s="14"/>
       <c r="E44" s="14"/>
       <c r="F44" s="13"/>
@@ -2245,7 +2359,7 @@
       <c r="K44" s="12"/>
       <c r="L44" s="9"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="45" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
         <v>51</v>
       </c>
@@ -2253,7 +2367,7 @@
         <v>63</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>63</v>
+        <v>235</v>
       </c>
       <c r="D45" s="14"/>
       <c r="E45" s="14"/>
@@ -2267,7 +2381,7 @@
       </c>
       <c r="L45" s="9"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="46" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
         <v>53</v>
       </c>
@@ -2275,7 +2389,7 @@
         <v>198</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>166</v>
+        <v>236</v>
       </c>
       <c r="D46" s="14"/>
       <c r="E46" s="14"/>
@@ -2289,7 +2403,7 @@
       </c>
       <c r="L46" s="9"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="47" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
         <v>80</v>
       </c>
@@ -2305,7 +2419,7 @@
       <c r="K47" s="15"/>
       <c r="L47" s="10"/>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="48" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
         <v>81</v>
       </c>
@@ -2313,7 +2427,7 @@
         <v>199</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>167</v>
+        <v>237</v>
       </c>
       <c r="D48" s="11"/>
       <c r="E48" s="11"/>
@@ -2329,7 +2443,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="49" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>82</v>
       </c>
@@ -2337,7 +2451,7 @@
         <v>200</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>168</v>
+        <v>238</v>
       </c>
       <c r="D49" s="14"/>
       <c r="E49" s="14"/>
@@ -2351,7 +2465,7 @@
       </c>
       <c r="L49" s="9"/>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="50" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>84</v>
       </c>
@@ -2359,7 +2473,7 @@
         <v>201</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>169</v>
+        <v>239</v>
       </c>
       <c r="D50" s="14"/>
       <c r="E50" s="14"/>
@@ -2373,7 +2487,7 @@
       </c>
       <c r="L50" s="9"/>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="51" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>85</v>
       </c>
@@ -2381,7 +2495,7 @@
         <v>202</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>170</v>
+        <v>240</v>
       </c>
       <c r="D51" s="14"/>
       <c r="E51" s="14"/>
@@ -2395,7 +2509,7 @@
       </c>
       <c r="L51" s="9"/>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="52" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
         <v>86</v>
       </c>
@@ -2403,7 +2517,7 @@
         <v>203</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>171</v>
+        <v>241</v>
       </c>
       <c r="D52" s="14"/>
       <c r="E52" s="14"/>
@@ -2417,7 +2531,7 @@
       </c>
       <c r="L52" s="9"/>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="53" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
         <v>87</v>
       </c>
@@ -2425,7 +2539,7 @@
         <v>204</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>172</v>
+        <v>242</v>
       </c>
       <c r="D53" s="14"/>
       <c r="E53" s="14"/>
@@ -2439,7 +2553,7 @@
       </c>
       <c r="L53" s="9"/>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="54" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
         <v>88</v>
       </c>
@@ -2447,7 +2561,7 @@
         <v>205</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>173</v>
+        <v>243</v>
       </c>
       <c r="D54" s="14"/>
       <c r="E54" s="14"/>
@@ -2461,7 +2575,7 @@
       </c>
       <c r="L54" s="9"/>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="55" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
         <v>90</v>
       </c>
@@ -2469,7 +2583,7 @@
         <v>206</v>
       </c>
       <c r="C55" s="11" t="s">
-        <v>174</v>
+        <v>244</v>
       </c>
       <c r="D55" s="14"/>
       <c r="E55" s="14"/>
@@ -2483,14 +2597,16 @@
       </c>
       <c r="L55" s="9"/>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="56" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
         <v>208</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>210</v>
       </c>
-      <c r="C56" s="11"/>
+      <c r="C56" s="11" t="s">
+        <v>245</v>
+      </c>
       <c r="D56" s="14"/>
       <c r="E56" s="14"/>
       <c r="F56" s="13"/>
@@ -2499,6 +2615,7 @@
       <c r="I56" s="13"/>
       <c r="J56" s="12"/>
       <c r="K56" s="12"/>
+      <c r="L56" s="0"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>